<commit_message>
Remodelação do planejamento com adição de um novo caso de uso
</commit_message>
<xml_diff>
--- a/6.Gerenciamento de Projeto/BRA - Planejamento e Controle do Projeto.xlsx
+++ b/6.Gerenciamento de Projeto/BRA - Planejamento e Controle do Projeto.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\fabioas\Documentos\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\fabioas\Development\bra-brasileirao_analyst\6.Gerenciamento de Projeto\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9FA6F68-5E84-4977-A1DB-1801D1C1471B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51661E92-8239-487E-B887-1507DF87717E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-19310" yWindow="-110" windowWidth="19420" windowHeight="11020" activeTab="3" xr2:uid="{31237A52-FFD1-4E1D-B5BB-391D11929C61}"/>
   </bookViews>
@@ -4738,7 +4738,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="352" uniqueCount="252">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="353" uniqueCount="253">
   <si>
     <t>Equipe</t>
   </si>
@@ -4835,9 +4835,6 @@
   </si>
   <si>
     <t>Planejar o Sprint</t>
-  </si>
-  <si>
-    <t>Estudar tecnologias</t>
   </si>
   <si>
     <t>Preparar Ambiente de Desenvolvimento</t>
@@ -5482,78 +5479,6 @@
     <t>Desenvolver Modelo de Objetos</t>
   </si>
   <si>
-    <t>Modelar solução para teste de arquitetura</t>
-  </si>
-  <si>
-    <t>Implementar funcionalidade para teste de arquitetura</t>
-  </si>
-  <si>
-    <t>Testar funcionalidade implementada</t>
-  </si>
-  <si>
-    <t>Projetar testes de funcionalidade</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Projetar testes para </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>UC 05 - Comparar clubes</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Modelar, Implementar e Testar o </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>UC 05 - Comparar clubes</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Projetar testes para </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>UC 04 - Favoritar atleta</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Modelar, Implementar e Testar o </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>UC 04 - Favoritar atleta</t>
-    </r>
-  </si>
-  <si>
     <r>
       <t xml:space="preserve">Projetar testes para </t>
     </r>
@@ -5630,6 +5555,51 @@
     <t>Em execução</t>
   </si>
   <si>
+    <t>Extrair dados dos clubes e dos atletas</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Implementar </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>UC 03 - Extrair dados dos clubes e dos atletas</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> para teste de arquitetura</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Testar </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>UC 03 - Extrair dados dos clubes e dos atletas</t>
+    </r>
+  </si>
+  <si>
+    <t>Refinar arquitetura</t>
+  </si>
+  <si>
     <r>
       <t xml:space="preserve">Projetar testes para </t>
     </r>
@@ -5641,7 +5611,7 @@
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
-      <t>UC 03 - Ver estatísticas do atleta</t>
+      <t>UC 04 - Ver estatísticas do atleta</t>
     </r>
   </si>
   <si>
@@ -5656,29 +5626,152 @@
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
-      <t>UC 03 - Ver estatísticas do atleta</t>
+      <t>UC 04 - Ver estatísticas do atleta</t>
     </r>
   </si>
   <si>
-    <t>Visão, modelo de caso de uso e plano de projeto</t>
-  </si>
-  <si>
-    <t>Histórias de usuário, modelo de objetos, modelos de arquitetura e UC 02</t>
-  </si>
-  <si>
-    <t>UC 03 e UC 05</t>
-  </si>
-  <si>
-    <t>UC 04 e UC 01</t>
-  </si>
-  <si>
-    <t>Guia de implantação, modelo de implantação, manual de suporte e treinamento e sistema em produção</t>
-  </si>
-  <si>
-    <t>Desenvolver Modelos de Arquitetura</t>
-  </si>
-  <si>
-    <t>Refinar arquiteturas</t>
+    <r>
+      <t xml:space="preserve">Projetar testes para </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>UC 06 - Comparar clubes</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Modelar, Implementar e Testar o </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>UC 06 - Comparar clubes</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Projetar testes para </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>UC 05 - Favoritar atleta</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Modelar, Implementar e Testar o </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>UC 05 - Favoritar atleta</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Modelar, Implementar e Testar o </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>UC 02 - Fazer login</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Projetar testes para </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>UC 02 - Fazer login</t>
+    </r>
+  </si>
+  <si>
+    <t>Desenvolver Modelo de Arquitetura</t>
+  </si>
+  <si>
+    <r>
+      <t>Modelar</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> UC 03 - Extrair dados dos clubes e dos atletas</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> para teste de arquitetura</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Projetar testes de </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>UC 03 - Extrair dados dos clubes e dos atletas</t>
+    </r>
+  </si>
+  <si>
+    <t>Visão, Modelo de Caso de Uso e plano de projeto</t>
+  </si>
+  <si>
+    <t>Histórias de Usuário, Modelo de Objetos, Modelo de Arquitetura, UC 03</t>
+  </si>
+  <si>
+    <t>UC 04 e UC 06</t>
+  </si>
+  <si>
+    <t>UC 05, UC 01 e UC 02, Guia de Implantação, Modelo de Implantação, Manual de Suporte e Treinamento e sistema em produção</t>
   </si>
 </sst>
 </file>
@@ -6558,6 +6651,79 @@
     <xf numFmtId="164" fontId="38" fillId="3" borderId="1" xfId="16" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="164" fontId="39" fillId="3" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="169" fontId="39" fillId="9" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="170" fontId="39" fillId="9" borderId="1" xfId="8" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="40" fillId="3" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="170" fontId="39" fillId="11" borderId="1" xfId="8" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="39" fillId="3" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="171" fontId="39" fillId="9" borderId="1" xfId="8" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="171" fontId="39" fillId="11" borderId="1" xfId="8" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="41" fillId="3" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="169" fontId="41" fillId="9" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="171" fontId="41" fillId="9" borderId="1" xfId="8" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="42" fillId="3" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="171" fontId="41" fillId="11" borderId="1" xfId="8" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="41" fillId="3" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="25" fillId="5" borderId="3" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="20" fillId="5" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="26" fillId="10" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="26" fillId="10" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="3" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="164" fontId="16" fillId="7" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -6577,29 +6743,10 @@
     <xf numFmtId="164" fontId="16" fillId="6" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="3" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="164" fontId="20" fillId="5" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="20" fillId="5" borderId="7" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="25" fillId="5" borderId="3" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="20" fillId="5" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="26" fillId="10" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="26" fillId="10" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="28" fillId="12" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -6660,60 +6807,6 @@
     </xf>
     <xf numFmtId="164" fontId="27" fillId="6" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="39" fillId="3" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="169" fontId="39" fillId="9" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="170" fontId="39" fillId="9" borderId="1" xfId="8" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="40" fillId="3" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="170" fontId="39" fillId="11" borderId="1" xfId="8" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="39" fillId="3" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="171" fontId="39" fillId="9" borderId="1" xfId="8" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="171" fontId="39" fillId="11" borderId="1" xfId="8" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="41" fillId="3" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="169" fontId="41" fillId="9" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="171" fontId="41" fillId="9" borderId="1" xfId="8" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="42" fillId="3" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="171" fontId="41" fillId="11" borderId="1" xfId="8" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="41" fillId="3" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="17">
@@ -6819,10 +6912,10 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>734450</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>162568</xdr:rowOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>314080</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>163838</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="3725997" cy="1047957"/>
     <xdr:pic>
@@ -6850,7 +6943,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="8379850" y="2346968"/>
+          <a:off x="7641980" y="2716538"/>
           <a:ext cx="3725997" cy="1047957"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -8612,18 +8705,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="20.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A1" s="122" t="s">
+      <c r="A1" s="134" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="122"/>
-      <c r="C1" s="122"/>
+      <c r="B1" s="134"/>
+      <c r="C1" s="134"/>
     </row>
     <row r="2" spans="1:3" ht="24.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="123" t="s">
-        <v>229</v>
-      </c>
-      <c r="B2" s="123"/>
-      <c r="C2" s="123"/>
+      <c r="A2" s="135" t="s">
+        <v>220</v>
+      </c>
+      <c r="B2" s="135"/>
+      <c r="C2" s="135"/>
     </row>
     <row r="3" spans="1:3" ht="15" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
@@ -8641,10 +8734,10 @@
         <v>4</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>233</v>
+        <v>224</v>
       </c>
       <c r="C4" s="115" t="s">
-        <v>230</v>
+        <v>221</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
@@ -8652,10 +8745,10 @@
         <v>5</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>234</v>
+        <v>225</v>
       </c>
       <c r="C5" s="115" t="s">
-        <v>231</v>
+        <v>222</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
@@ -8663,10 +8756,10 @@
         <v>6</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>235</v>
+        <v>226</v>
       </c>
       <c r="C6" s="115" t="s">
-        <v>232</v>
+        <v>223</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
@@ -8743,7 +8836,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F6C5642-BF97-4AFF-B370-04CC3D024494}">
-  <dimension ref="A1:AMJ48"/>
+  <dimension ref="A1:AMJ49"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.19921875" style="21" customWidth="1"/>
@@ -8752,7 +8845,7 @@
     <col min="4" max="4" width="8.69921875" style="19" customWidth="1"/>
     <col min="5" max="5" width="1.59765625" style="4" customWidth="1"/>
     <col min="6" max="6" width="4.19921875" style="4" customWidth="1"/>
-    <col min="7" max="7" width="18.8984375" style="4" customWidth="1"/>
+    <col min="7" max="7" width="26.3984375" style="4" bestFit="1" customWidth="1"/>
     <col min="8" max="9" width="8.5" style="4" customWidth="1"/>
     <col min="10" max="10" width="10.69921875" style="4" customWidth="1"/>
     <col min="11" max="11" width="11.8984375" style="4" customWidth="1"/>
@@ -8761,38 +8854,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="137" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="F1" s="118" t="s">
+      <c r="B1" s="137"/>
+      <c r="C1" s="137"/>
+      <c r="D1" s="137"/>
+      <c r="F1" s="138" t="s">
         <v>8</v>
       </c>
-      <c r="G1" s="118"/>
-      <c r="H1" s="118"/>
-      <c r="I1" s="118"/>
-      <c r="J1" s="118"/>
-      <c r="K1" s="118"/>
-      <c r="L1" s="118"/>
+      <c r="G1" s="138"/>
+      <c r="H1" s="138"/>
+      <c r="I1" s="138"/>
+      <c r="J1" s="138"/>
+      <c r="K1" s="138"/>
+      <c r="L1" s="138"/>
     </row>
     <row r="2" spans="1:12" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="119" t="s">
+      <c r="A2" s="139" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="119"/>
-      <c r="C2" s="119"/>
-      <c r="D2" s="119"/>
-      <c r="F2" s="120" t="s">
+      <c r="B2" s="139"/>
+      <c r="C2" s="139"/>
+      <c r="D2" s="139"/>
+      <c r="F2" s="140" t="s">
         <v>10</v>
       </c>
-      <c r="G2" s="120"/>
-      <c r="H2" s="120"/>
-      <c r="I2" s="120"/>
-      <c r="J2" s="120"/>
-      <c r="K2" s="120"/>
-      <c r="L2" s="120"/>
+      <c r="G2" s="140"/>
+      <c r="H2" s="140"/>
+      <c r="I2" s="140"/>
+      <c r="J2" s="140"/>
+      <c r="K2" s="140"/>
+      <c r="L2" s="140"/>
     </row>
     <row r="3" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
@@ -8813,20 +8906,20 @@
       <c r="G3" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="H3" s="121" t="s">
+      <c r="H3" s="141" t="s">
         <v>8</v>
       </c>
-      <c r="I3" s="121"/>
-      <c r="J3" s="121"/>
-      <c r="K3" s="121"/>
-      <c r="L3" s="121"/>
+      <c r="I3" s="141"/>
+      <c r="J3" s="141"/>
+      <c r="K3" s="141"/>
+      <c r="L3" s="141"/>
     </row>
     <row r="4" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="116" t="s">
+      <c r="A4" s="136" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="116"/>
-      <c r="C4" s="116"/>
+      <c r="B4" s="136"/>
+      <c r="C4" s="136"/>
       <c r="D4" s="8" t="s">
         <v>17</v>
       </c>
@@ -8869,13 +8962,13 @@
         <v>1</v>
       </c>
       <c r="G5" s="12" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="H5" s="15">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I5" s="15">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J5" s="15">
         <v>0</v>
@@ -8885,7 +8978,7 @@
       </c>
       <c r="L5" s="16">
         <f>SUM(H5:K5)</f>
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="6" spans="1:12" ht="13.8" x14ac:dyDescent="0.25">
@@ -8905,13 +8998,13 @@
         <v>2</v>
       </c>
       <c r="G6" s="12" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="H6" s="15">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I6" s="15">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J6" s="15">
         <v>0</v>
@@ -8921,7 +9014,7 @@
       </c>
       <c r="L6" s="16">
         <f>SUM(H6:K6)</f>
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="7" spans="1:12" ht="13.8" x14ac:dyDescent="0.25">
@@ -8935,16 +9028,16 @@
         <v>27</v>
       </c>
       <c r="D7" s="13">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F7" s="14">
         <v>3</v>
       </c>
       <c r="G7" s="12" t="s">
-        <v>213</v>
+        <v>234</v>
       </c>
       <c r="H7" s="15">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="I7" s="15">
         <v>8</v>
@@ -8953,11 +9046,11 @@
         <v>10</v>
       </c>
       <c r="K7" s="15">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="L7" s="16">
         <f t="shared" ref="L7:L9" si="0">SUM(H7:K7)</f>
-        <v>37</v>
+        <v>33</v>
       </c>
     </row>
     <row r="8" spans="1:12" ht="13.8" x14ac:dyDescent="0.25">
@@ -8971,29 +9064,29 @@
         <v>28</v>
       </c>
       <c r="D8" s="13">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F8" s="14">
         <v>4</v>
       </c>
       <c r="G8" s="12" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="H8" s="15">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="I8" s="15">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J8" s="15">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K8" s="15">
         <v>6</v>
       </c>
       <c r="L8" s="16">
         <f t="shared" si="0"/>
-        <v>17</v>
+        <v>31</v>
       </c>
     </row>
     <row r="9" spans="1:12" ht="13.8" x14ac:dyDescent="0.25">
@@ -9004,32 +9097,32 @@
         <v>16</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D9" s="13">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="F9" s="17">
         <v>5</v>
       </c>
       <c r="G9" s="12" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="H9" s="15">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="I9" s="15">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="J9" s="15">
         <v>0</v>
       </c>
       <c r="K9" s="15">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="L9" s="16">
         <f t="shared" si="0"/>
-        <v>29</v>
+        <v>14</v>
       </c>
     </row>
     <row r="10" spans="1:12" ht="13.8" x14ac:dyDescent="0.25">
@@ -9043,25 +9136,40 @@
         <v>29</v>
       </c>
       <c r="D10" s="13">
-        <v>2</v>
-      </c>
-      <c r="F10"/>
-      <c r="G10"/>
-      <c r="H10"/>
-      <c r="I10"/>
-      <c r="J10"/>
-      <c r="K10"/>
-      <c r="L10"/>
+        <v>1</v>
+      </c>
+      <c r="F10" s="17">
+        <v>6</v>
+      </c>
+      <c r="G10" s="12" t="s">
+        <v>214</v>
+      </c>
+      <c r="H10" s="15">
+        <v>9</v>
+      </c>
+      <c r="I10" s="15">
+        <v>6</v>
+      </c>
+      <c r="J10" s="15">
+        <v>0</v>
+      </c>
+      <c r="K10" s="15">
+        <v>7</v>
+      </c>
+      <c r="L10" s="16">
+        <f t="shared" ref="L10" si="1">SUM(H10:K10)</f>
+        <v>22</v>
+      </c>
     </row>
     <row r="11" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="116" t="s">
+      <c r="A11" s="136" t="s">
         <v>30</v>
       </c>
-      <c r="B11" s="116"/>
-      <c r="C11" s="116"/>
+      <c r="B11" s="136"/>
+      <c r="C11" s="136"/>
       <c r="D11" s="8">
         <f>SUM(D5:D10)</f>
-        <v>9</v>
+        <v>10.5</v>
       </c>
       <c r="F11"/>
       <c r="G11"/>
@@ -9100,10 +9208,10 @@
         <v>30</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D13" s="13">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="F13"/>
       <c r="G13"/>
@@ -9115,16 +9223,16 @@
     </row>
     <row r="14" spans="1:12" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A14" s="10">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B14" s="11" t="s">
         <v>30</v>
       </c>
       <c r="C14" s="12" t="s">
-        <v>32</v>
+        <v>216</v>
       </c>
       <c r="D14" s="13">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="F14"/>
       <c r="G14"/>
@@ -9136,16 +9244,16 @@
     </row>
     <row r="15" spans="1:12" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A15" s="10">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B15" s="11" t="s">
         <v>30</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>217</v>
+        <v>246</v>
       </c>
       <c r="D15" s="13">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="F15"/>
       <c r="G15"/>
@@ -9157,16 +9265,16 @@
     </row>
     <row r="16" spans="1:12" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A16" s="10">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B16" s="11" t="s">
         <v>30</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="D16" s="13">
-        <v>8</v>
+        <v>0.5</v>
       </c>
       <c r="F16"/>
       <c r="G16"/>
@@ -9178,16 +9286,16 @@
     </row>
     <row r="17" spans="1:12" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A17" s="10">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B17" s="11" t="s">
         <v>30</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>218</v>
+        <v>248</v>
       </c>
       <c r="D17" s="13">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="F17"/>
       <c r="G17"/>
@@ -9199,16 +9307,16 @@
     </row>
     <row r="18" spans="1:12" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A18" s="10">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B18" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="C18" s="12" t="s">
-        <v>221</v>
+      <c r="C18" s="18" t="s">
+        <v>32</v>
       </c>
       <c r="D18" s="13">
-        <v>2</v>
+        <v>0.5</v>
       </c>
       <c r="F18"/>
       <c r="G18"/>
@@ -9220,16 +9328,16 @@
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" s="10">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B19" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="C19" s="18" t="s">
-        <v>33</v>
+      <c r="C19" s="12" t="s">
+        <v>235</v>
       </c>
       <c r="D19" s="13">
-        <v>0.5</v>
+        <v>8</v>
       </c>
       <c r="H19" s="19"/>
       <c r="I19" s="19"/>
@@ -9239,16 +9347,16 @@
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" s="10">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B20" s="11" t="s">
         <v>30</v>
       </c>
       <c r="C20" s="12" t="s">
-        <v>219</v>
+        <v>236</v>
       </c>
       <c r="D20" s="13">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H20" s="19"/>
       <c r="I20" s="19"/>
@@ -9258,16 +9366,16 @@
     </row>
     <row r="21" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="10">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B21" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="C21" s="12" t="s">
-        <v>220</v>
+      <c r="C21" s="18" t="s">
+        <v>237</v>
       </c>
       <c r="D21" s="13">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H21" s="19"/>
       <c r="I21" s="19"/>
@@ -9277,16 +9385,16 @@
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" s="10">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B22" s="11" t="s">
         <v>30</v>
       </c>
       <c r="C22" s="18" t="s">
-        <v>251</v>
+        <v>33</v>
       </c>
       <c r="D22" s="13">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="H22" s="19"/>
       <c r="I22" s="19"/>
@@ -9296,7 +9404,7 @@
     </row>
     <row r="23" spans="1:12" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A23" s="10">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B23" s="11" t="s">
         <v>30</v>
@@ -9309,39 +9417,39 @@
       </c>
     </row>
     <row r="24" spans="1:12" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A24" s="10">
-        <v>19</v>
-      </c>
-      <c r="B24" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="C24" s="18" t="s">
+      <c r="A24" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="D24" s="13">
-        <v>2</v>
+      <c r="B24" s="7"/>
+      <c r="C24" s="7"/>
+      <c r="D24" s="8">
+        <f>SUM(D12:D23)</f>
+        <v>30.5</v>
       </c>
     </row>
     <row r="25" spans="1:12" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A25" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="B25" s="7"/>
-      <c r="C25" s="7"/>
-      <c r="D25" s="8">
-        <f>SUM(D12:D24)</f>
-        <v>56</v>
+      <c r="A25" s="10">
+        <v>20</v>
+      </c>
+      <c r="B25" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="C25" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="D25" s="13">
+        <v>1</v>
       </c>
     </row>
     <row r="26" spans="1:12" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A26" s="10">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B26" s="11" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C26" s="12" t="s">
-        <v>31</v>
+        <v>238</v>
       </c>
       <c r="D26" s="13">
         <v>1</v>
@@ -9349,100 +9457,100 @@
     </row>
     <row r="27" spans="1:12" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A27" s="10">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B27" s="11" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C27" s="12" t="s">
-        <v>243</v>
+        <v>239</v>
       </c>
       <c r="D27" s="13">
-        <v>2</v>
+        <v>20</v>
       </c>
     </row>
     <row r="28" spans="1:12" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A28" s="10">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B28" s="11" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C28" s="12" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="D28" s="13">
-        <v>20</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29" spans="1:12" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A29" s="10">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B29" s="11" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C29" s="12" t="s">
-        <v>222</v>
+        <v>241</v>
       </c>
       <c r="D29" s="13">
-        <v>2</v>
+        <v>20</v>
       </c>
     </row>
     <row r="30" spans="1:12" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A30" s="10">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B30" s="11" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C30" s="12" t="s">
-        <v>223</v>
+        <v>242</v>
       </c>
       <c r="D30" s="13">
-        <v>20</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="10">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B31" s="11" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C31" s="12" t="s">
-        <v>224</v>
+        <v>243</v>
       </c>
       <c r="D31" s="13">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="32" spans="1:12" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A32" s="10">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B32" s="11" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C32" s="12" t="s">
-        <v>225</v>
+        <v>217</v>
       </c>
       <c r="D32" s="13">
-        <v>13</v>
+        <v>2</v>
       </c>
     </row>
     <row r="33" spans="1:4" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A33" s="10">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B33" s="11" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C33" s="12" t="s">
-        <v>226</v>
+        <v>218</v>
       </c>
       <c r="D33" s="13">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="34" spans="1:4" ht="13.8" x14ac:dyDescent="0.25">
@@ -9450,77 +9558,77 @@
         <v>26</v>
       </c>
       <c r="B34" s="11" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C34" s="12" t="s">
-        <v>227</v>
+        <v>245</v>
       </c>
       <c r="D34" s="13">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="35" spans="1:4" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A35" s="10">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="B35" s="11" t="s">
-        <v>36</v>
-      </c>
-      <c r="C35" s="18" t="s">
-        <v>34</v>
+        <v>35</v>
+      </c>
+      <c r="C35" s="12" t="s">
+        <v>244</v>
       </c>
       <c r="D35" s="13">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="36" spans="1:4" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A36" s="10">
+        <v>29</v>
+      </c>
+      <c r="B36" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="C36" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="D36" s="13">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A37" s="10">
         <v>30</v>
       </c>
-      <c r="B36" s="11" t="s">
+      <c r="B37" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="C37" s="18" t="s">
+        <v>34</v>
+      </c>
+      <c r="D37" s="13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A38" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="C36" s="18" t="s">
-        <v>35</v>
-      </c>
-      <c r="D36" s="13">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A37" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="B37" s="7"/>
-      <c r="C37" s="7"/>
-      <c r="D37" s="8">
-        <f>SUM(D26:D36)</f>
-        <v>73</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A38" s="10">
-        <v>31</v>
-      </c>
-      <c r="B38" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="C38" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="D38" s="13">
-        <v>1</v>
+      <c r="B38" s="7"/>
+      <c r="C38" s="7"/>
+      <c r="D38" s="8">
+        <f>SUM(D25:D37)</f>
+        <v>70.5</v>
       </c>
     </row>
     <row r="39" spans="1:4" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A39" s="10">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B39" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="C39" s="18" t="s">
-        <v>38</v>
+        <v>36</v>
+      </c>
+      <c r="C39" s="12" t="s">
+        <v>31</v>
       </c>
       <c r="D39" s="13">
         <v>1</v>
@@ -9528,13 +9636,13 @@
     </row>
     <row r="40" spans="1:4" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A40" s="10">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B40" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="C40" s="18" t="s">
         <v>37</v>
-      </c>
-      <c r="C40" s="18" t="s">
-        <v>39</v>
       </c>
       <c r="D40" s="13">
         <v>2</v>
@@ -9542,101 +9650,115 @@
     </row>
     <row r="41" spans="1:4" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="10">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B41" s="11" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C41" s="18" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="D41" s="13">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="42" spans="1:4" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A42" s="10">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B42" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="C42" s="12" t="s">
-        <v>228</v>
+        <v>36</v>
+      </c>
+      <c r="C42" s="18" t="s">
+        <v>39</v>
       </c>
       <c r="D42" s="13">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="43" spans="1:4" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A43" s="10">
+        <v>35</v>
+      </c>
+      <c r="B43" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="B43" s="11" t="s">
-        <v>37</v>
-      </c>
       <c r="C43" s="12" t="s">
-        <v>41</v>
+        <v>219</v>
       </c>
       <c r="D43" s="13">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="44" spans="1:4" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A44" s="10">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B44" s="11" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C44" s="12" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D44" s="13">
-        <v>13</v>
+        <v>3</v>
       </c>
     </row>
     <row r="45" spans="1:4" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A45" s="10">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B45" s="11" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C45" s="12" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D45" s="13">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="46" spans="1:4" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A46" s="10">
-        <v>39</v>
-      </c>
-      <c r="B46" s="20" t="s">
-        <v>37</v>
-      </c>
-      <c r="C46" s="18" t="s">
-        <v>34</v>
+        <v>38</v>
+      </c>
+      <c r="B46" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="C46" s="12" t="s">
+        <v>42</v>
       </c>
       <c r="D46" s="13">
         <v>1</v>
       </c>
     </row>
     <row r="47" spans="1:4" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A47" s="23"/>
-      <c r="B47" s="23"/>
-      <c r="C47" s="23"/>
-      <c r="D47" s="8">
-        <f>SUM(D38:D46)</f>
-        <v>32</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" ht="15.6" x14ac:dyDescent="0.25">
-      <c r="D48" s="22">
-        <f>SUM(D11,D25,D37,D47)</f>
-        <v>170</v>
+      <c r="A47" s="10">
+        <v>39</v>
+      </c>
+      <c r="B47" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="C47" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="D47" s="13">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A48" s="23"/>
+      <c r="B48" s="23"/>
+      <c r="C48" s="23"/>
+      <c r="D48" s="8">
+        <f>SUM(D39:D47)</f>
+        <v>18.5</v>
+      </c>
+    </row>
+    <row r="49" spans="4:4" ht="15.6" x14ac:dyDescent="0.25">
+      <c r="D49" s="22">
+        <f>SUM(D11,D24,D38,D48)</f>
+        <v>130</v>
       </c>
     </row>
   </sheetData>
@@ -9670,49 +9792,49 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A1" s="124" t="s">
-        <v>44</v>
-      </c>
-      <c r="B1" s="124"/>
-      <c r="C1" s="124"/>
+      <c r="A1" s="142" t="s">
+        <v>43</v>
+      </c>
+      <c r="B1" s="142"/>
+      <c r="C1" s="142"/>
     </row>
     <row r="2" spans="1:5" ht="7.5" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="3" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A3" s="125" t="s">
-        <v>45</v>
-      </c>
-      <c r="B3" s="125"/>
-      <c r="C3" s="125"/>
+      <c r="A3" s="143" t="s">
+        <v>44</v>
+      </c>
+      <c r="B3" s="143"/>
+      <c r="C3" s="143"/>
     </row>
     <row r="4" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A4" s="25" t="s">
+        <v>45</v>
+      </c>
+      <c r="B4" s="26">
+        <f>Backlog_Produto!$D$49</f>
+        <v>130</v>
+      </c>
+      <c r="C4" s="25" t="s">
         <v>46</v>
-      </c>
-      <c r="B4" s="26">
-        <f>Backlog_Produto!$D$48</f>
-        <v>170</v>
-      </c>
-      <c r="C4" s="25" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="27" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B5" s="28">
         <v>0.6</v>
       </c>
       <c r="C5" s="27" t="s">
+        <v>48</v>
+      </c>
+      <c r="E5" s="1" t="s">
         <v>49</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="29" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B6" s="30">
         <v>3</v>
@@ -9721,85 +9843,85 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="29" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B7" s="30">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C7" s="29" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="29" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B8" s="31">
         <f>B6*B7*2</f>
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="C8" s="29" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="19.8" x14ac:dyDescent="0.4">
       <c r="A9" s="32" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B9" s="33">
         <f>B11/2</f>
-        <v>5.0370370370370372</v>
+        <v>4.333333333333333</v>
       </c>
       <c r="C9" s="32" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="19.8" x14ac:dyDescent="0.4">
       <c r="A10" s="34" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B10" s="33">
         <f>B4+(B4*B5)</f>
-        <v>272</v>
+        <v>208</v>
       </c>
       <c r="C10" s="34" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" s="29" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B11" s="31">
         <f>B10/B8*2</f>
-        <v>10.074074074074074</v>
+        <v>8.6666666666666661</v>
       </c>
       <c r="C11" s="29" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A12" s="25" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B12" s="35">
         <f>B11/4</f>
-        <v>2.5185185185185186</v>
+        <v>2.1666666666666665</v>
       </c>
       <c r="C12" s="25" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A14" s="143" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A14" s="125" t="s">
-        <v>61</v>
-      </c>
-      <c r="B14" s="125"/>
-      <c r="C14" s="125"/>
+      <c r="B14" s="143"/>
+      <c r="C14" s="143"/>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" s="29" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B15" s="36">
         <v>15</v>
@@ -9808,17 +9930,17 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" s="29" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B16" s="38">
         <f>B10*B15</f>
-        <v>4080</v>
+        <v>3120</v>
       </c>
       <c r="C16" s="37"/>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" s="29" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B17" s="28">
         <v>0.2</v>
@@ -9827,27 +9949,27 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="29" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B18" s="39">
         <f>B16*B17</f>
-        <v>816</v>
+        <v>624</v>
       </c>
       <c r="C18" s="37"/>
     </row>
     <row r="19" spans="1:3" ht="18" x14ac:dyDescent="0.35">
       <c r="A19" s="40" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B19" s="41">
         <f>B16+B18</f>
-        <v>4896</v>
+        <v>3744</v>
       </c>
       <c r="C19" s="37"/>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" s="29" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B20" s="28">
         <v>0.2</v>
@@ -9856,21 +9978,21 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" s="29" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B21" s="42">
         <f>B19*B20</f>
-        <v>979.2</v>
+        <v>748.80000000000007</v>
       </c>
       <c r="C21" s="37"/>
     </row>
     <row r="22" spans="1:3" ht="18" x14ac:dyDescent="0.35">
       <c r="A22" s="40" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B22" s="41">
         <f>B19+B21</f>
-        <v>5875.2</v>
+        <v>4492.8</v>
       </c>
       <c r="C22" s="37"/>
     </row>
@@ -9904,295 +10026,291 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="23.4" x14ac:dyDescent="0.45">
-      <c r="A1" s="126" t="s">
+      <c r="A1" s="130" t="s">
+        <v>69</v>
+      </c>
+      <c r="B1" s="130"/>
+      <c r="C1" s="130"/>
+      <c r="D1" s="130"/>
+      <c r="E1" s="130"/>
+      <c r="F1" s="130"/>
+      <c r="G1" s="130"/>
+      <c r="H1" s="130"/>
+      <c r="I1" s="130"/>
+      <c r="J1" s="130"/>
+      <c r="K1" s="130"/>
+    </row>
+    <row r="2" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="131" t="s">
         <v>70</v>
       </c>
-      <c r="B1" s="126"/>
-      <c r="C1" s="126"/>
-      <c r="D1" s="126"/>
-      <c r="E1" s="126"/>
-      <c r="F1" s="126"/>
-      <c r="G1" s="126"/>
-      <c r="H1" s="126"/>
-      <c r="I1" s="126"/>
-      <c r="J1" s="126"/>
-      <c r="K1" s="126"/>
-    </row>
-    <row r="2" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="127" t="s">
-        <v>71</v>
-      </c>
-      <c r="B2" s="127"/>
-      <c r="C2" s="127"/>
-      <c r="D2" s="127"/>
+      <c r="B2" s="131"/>
+      <c r="C2" s="131"/>
+      <c r="D2" s="131"/>
       <c r="E2" s="43">
         <f>Planejamento!$B$10</f>
-        <v>272</v>
+        <v>208</v>
       </c>
       <c r="F2" s="44"/>
-      <c r="G2" s="127" t="s">
-        <v>71</v>
-      </c>
-      <c r="H2" s="127"/>
-      <c r="I2" s="127"/>
-      <c r="J2" s="127"/>
+      <c r="G2" s="131" t="s">
+        <v>70</v>
+      </c>
+      <c r="H2" s="131"/>
+      <c r="I2" s="131"/>
+      <c r="J2" s="131"/>
       <c r="K2" s="43"/>
     </row>
     <row r="3" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A3" s="45"/>
       <c r="B3" s="46"/>
-      <c r="C3" s="128" t="s">
+      <c r="C3" s="132" t="s">
+        <v>71</v>
+      </c>
+      <c r="D3" s="132"/>
+      <c r="E3" s="132"/>
+      <c r="F3" s="47"/>
+      <c r="G3" s="133" t="s">
         <v>72</v>
       </c>
-      <c r="D3" s="128"/>
-      <c r="E3" s="128"/>
-      <c r="F3" s="47"/>
-      <c r="G3" s="129" t="s">
-        <v>73</v>
-      </c>
-      <c r="H3" s="129"/>
-      <c r="I3" s="129"/>
+      <c r="H3" s="133"/>
+      <c r="I3" s="133"/>
       <c r="J3" s="49"/>
       <c r="K3" s="50"/>
     </row>
     <row r="4" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A4" s="48" t="s">
+        <v>73</v>
+      </c>
+      <c r="B4" s="48" t="s">
         <v>74</v>
       </c>
-      <c r="B4" s="48" t="s">
+      <c r="C4" s="48" t="s">
         <v>75</v>
       </c>
-      <c r="C4" s="48" t="s">
+      <c r="D4" s="48" t="s">
         <v>76</v>
-      </c>
-      <c r="D4" s="48" t="s">
-        <v>77</v>
       </c>
       <c r="E4" s="48" t="s">
         <v>17</v>
       </c>
       <c r="F4" s="48" t="s">
+        <v>77</v>
+      </c>
+      <c r="G4" s="48" t="s">
+        <v>75</v>
+      </c>
+      <c r="H4" s="48" t="s">
         <v>78</v>
-      </c>
-      <c r="G4" s="48" t="s">
-        <v>76</v>
-      </c>
-      <c r="H4" s="48" t="s">
-        <v>79</v>
       </c>
       <c r="I4" s="48" t="s">
         <v>17</v>
       </c>
       <c r="J4" s="51" t="s">
+        <v>79</v>
+      </c>
+      <c r="K4" s="48" t="s">
         <v>80</v>
-      </c>
-      <c r="K4" s="48" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A5" s="52">
         <v>1</v>
       </c>
-      <c r="B5" s="151" t="s">
-        <v>245</v>
-      </c>
-      <c r="C5" s="152">
+      <c r="B5" s="116" t="s">
+        <v>249</v>
+      </c>
+      <c r="C5" s="117">
         <v>46252</v>
       </c>
-      <c r="D5" s="152">
-        <v>46235</v>
-      </c>
-      <c r="E5" s="153">
-        <v>9</v>
-      </c>
-      <c r="F5" s="154" t="s">
-        <v>242</v>
-      </c>
-      <c r="G5" s="152">
+      <c r="D5" s="117">
+        <v>46266</v>
+      </c>
+      <c r="E5" s="118">
+        <v>10.5</v>
+      </c>
+      <c r="F5" s="119" t="s">
+        <v>233</v>
+      </c>
+      <c r="G5" s="117">
         <v>46252</v>
       </c>
-      <c r="H5" s="152"/>
-      <c r="I5" s="153"/>
-      <c r="J5" s="155"/>
-      <c r="K5" s="156" t="s">
-        <v>241</v>
+      <c r="H5" s="117">
+        <v>46259</v>
+      </c>
+      <c r="I5" s="118">
+        <v>5</v>
+      </c>
+      <c r="J5" s="120">
+        <v>-5.5</v>
+      </c>
+      <c r="K5" s="121" t="s">
+        <v>232</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A6" s="52">
         <v>2</v>
       </c>
-      <c r="B6" s="151" t="s">
-        <v>246</v>
-      </c>
-      <c r="C6" s="152">
+      <c r="B6" s="116" t="s">
+        <v>250</v>
+      </c>
+      <c r="C6" s="117">
         <v>46273</v>
       </c>
-      <c r="D6" s="152">
+      <c r="D6" s="117">
         <v>46287</v>
       </c>
-      <c r="E6" s="157">
-        <v>54</v>
-      </c>
-      <c r="F6" s="154" t="s">
-        <v>82</v>
-      </c>
-      <c r="G6" s="152"/>
-      <c r="H6" s="152"/>
-      <c r="I6" s="157"/>
-      <c r="J6" s="158"/>
-      <c r="K6" s="156"/>
+      <c r="E6" s="122">
+        <v>30.5</v>
+      </c>
+      <c r="F6" s="119" t="s">
+        <v>81</v>
+      </c>
+      <c r="G6" s="117"/>
+      <c r="H6" s="117"/>
+      <c r="I6" s="122"/>
+      <c r="J6" s="123"/>
+      <c r="K6" s="121"/>
     </row>
     <row r="7" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A7" s="52">
         <v>3</v>
       </c>
-      <c r="B7" s="151" t="s">
-        <v>247</v>
-      </c>
-      <c r="C7" s="152">
+      <c r="B7" s="116" t="s">
+        <v>251</v>
+      </c>
+      <c r="C7" s="117">
         <v>46294</v>
       </c>
-      <c r="D7" s="152">
+      <c r="D7" s="117">
         <v>46308</v>
       </c>
-      <c r="E7" s="157">
-        <v>47</v>
-      </c>
-      <c r="F7" s="154" t="s">
-        <v>82</v>
-      </c>
-      <c r="G7" s="152"/>
-      <c r="H7" s="152"/>
-      <c r="I7" s="157"/>
-      <c r="J7" s="158"/>
-      <c r="K7" s="156"/>
-    </row>
-    <row r="8" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="E7" s="122">
+        <v>43</v>
+      </c>
+      <c r="F7" s="119" t="s">
+        <v>81</v>
+      </c>
+      <c r="G7" s="117"/>
+      <c r="H7" s="117"/>
+      <c r="I7" s="122"/>
+      <c r="J7" s="123"/>
+      <c r="K7" s="121"/>
+    </row>
+    <row r="8" spans="1:11" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A8" s="52">
         <v>4</v>
       </c>
-      <c r="B8" s="159" t="s">
-        <v>248</v>
-      </c>
-      <c r="C8" s="160">
+      <c r="B8" s="124" t="s">
+        <v>252</v>
+      </c>
+      <c r="C8" s="125">
         <v>46315</v>
       </c>
-      <c r="D8" s="160">
+      <c r="D8" s="125">
         <v>46329</v>
       </c>
-      <c r="E8" s="161">
-        <v>28</v>
-      </c>
-      <c r="F8" s="162" t="s">
-        <v>82</v>
-      </c>
-      <c r="G8" s="160"/>
-      <c r="H8" s="160"/>
-      <c r="I8" s="161"/>
-      <c r="J8" s="163"/>
-      <c r="K8" s="164"/>
-    </row>
-    <row r="9" spans="1:11" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="E8" s="126">
+        <v>46</v>
+      </c>
+      <c r="F8" s="127" t="s">
+        <v>81</v>
+      </c>
+      <c r="G8" s="125"/>
+      <c r="H8" s="125"/>
+      <c r="I8" s="126"/>
+      <c r="J8" s="128"/>
+      <c r="K8" s="129"/>
+    </row>
+    <row r="9" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A9" s="52">
         <v>5</v>
       </c>
-      <c r="B9" s="159" t="s">
-        <v>249</v>
-      </c>
-      <c r="C9" s="160">
-        <v>46336</v>
-      </c>
-      <c r="D9" s="160">
-        <v>46350</v>
-      </c>
-      <c r="E9" s="161">
-        <v>32</v>
-      </c>
-      <c r="F9" s="162" t="s">
-        <v>82</v>
-      </c>
-      <c r="G9" s="160"/>
-      <c r="H9" s="160"/>
-      <c r="I9" s="161"/>
-      <c r="J9" s="163"/>
-      <c r="K9" s="164"/>
+      <c r="B9" s="124"/>
+      <c r="C9" s="125"/>
+      <c r="D9" s="125"/>
+      <c r="E9" s="126"/>
+      <c r="F9" s="127"/>
+      <c r="G9" s="125"/>
+      <c r="H9" s="125"/>
+      <c r="I9" s="126"/>
+      <c r="J9" s="128"/>
+      <c r="K9" s="129"/>
     </row>
     <row r="10" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A10" s="52">
         <v>6</v>
       </c>
-      <c r="B10" s="159"/>
-      <c r="C10" s="160"/>
-      <c r="D10" s="160"/>
-      <c r="E10" s="161"/>
-      <c r="F10" s="162"/>
-      <c r="G10" s="160"/>
-      <c r="H10" s="160"/>
-      <c r="I10" s="161"/>
-      <c r="J10" s="163"/>
-      <c r="K10" s="164"/>
+      <c r="B10" s="124"/>
+      <c r="C10" s="125"/>
+      <c r="D10" s="125"/>
+      <c r="E10" s="126"/>
+      <c r="F10" s="127"/>
+      <c r="G10" s="125"/>
+      <c r="H10" s="125"/>
+      <c r="I10" s="126"/>
+      <c r="J10" s="128"/>
+      <c r="K10" s="129"/>
     </row>
     <row r="11" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A11" s="52">
         <v>7</v>
       </c>
-      <c r="B11" s="159"/>
-      <c r="C11" s="160"/>
-      <c r="D11" s="160"/>
-      <c r="E11" s="161"/>
-      <c r="F11" s="162"/>
-      <c r="G11" s="160"/>
-      <c r="H11" s="160"/>
-      <c r="I11" s="161"/>
-      <c r="J11" s="163"/>
-      <c r="K11" s="164"/>
+      <c r="B11" s="124"/>
+      <c r="C11" s="125"/>
+      <c r="D11" s="125"/>
+      <c r="E11" s="126"/>
+      <c r="F11" s="127"/>
+      <c r="G11" s="125"/>
+      <c r="H11" s="125"/>
+      <c r="I11" s="126"/>
+      <c r="J11" s="128"/>
+      <c r="K11" s="129"/>
     </row>
     <row r="12" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A12" s="52">
         <v>8</v>
       </c>
-      <c r="B12" s="159"/>
-      <c r="C12" s="160"/>
-      <c r="D12" s="160"/>
-      <c r="E12" s="161"/>
-      <c r="F12" s="162"/>
-      <c r="G12" s="160"/>
-      <c r="H12" s="160"/>
-      <c r="I12" s="161"/>
-      <c r="J12" s="163"/>
-      <c r="K12" s="164"/>
+      <c r="B12" s="124"/>
+      <c r="C12" s="125"/>
+      <c r="D12" s="125"/>
+      <c r="E12" s="126"/>
+      <c r="F12" s="127"/>
+      <c r="G12" s="125"/>
+      <c r="H12" s="125"/>
+      <c r="I12" s="126"/>
+      <c r="J12" s="128"/>
+      <c r="K12" s="129"/>
     </row>
     <row r="13" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A13" s="52">
         <v>9</v>
       </c>
-      <c r="B13" s="159"/>
-      <c r="C13" s="160"/>
-      <c r="D13" s="160"/>
-      <c r="E13" s="161"/>
-      <c r="F13" s="162"/>
-      <c r="G13" s="160"/>
-      <c r="H13" s="160"/>
-      <c r="I13" s="161"/>
-      <c r="J13" s="163"/>
-      <c r="K13" s="164"/>
+      <c r="B13" s="124"/>
+      <c r="C13" s="125"/>
+      <c r="D13" s="125"/>
+      <c r="E13" s="126"/>
+      <c r="F13" s="127"/>
+      <c r="G13" s="125"/>
+      <c r="H13" s="125"/>
+      <c r="I13" s="126"/>
+      <c r="J13" s="128"/>
+      <c r="K13" s="129"/>
     </row>
     <row r="14" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A14" s="52">
         <v>10</v>
       </c>
-      <c r="B14" s="159"/>
-      <c r="C14" s="160"/>
-      <c r="D14" s="160"/>
-      <c r="E14" s="161"/>
-      <c r="F14" s="162"/>
-      <c r="G14" s="160"/>
-      <c r="H14" s="160"/>
-      <c r="I14" s="161"/>
-      <c r="J14" s="163"/>
-      <c r="K14" s="164"/>
+      <c r="B14" s="124"/>
+      <c r="C14" s="125"/>
+      <c r="D14" s="125"/>
+      <c r="E14" s="126"/>
+      <c r="F14" s="127"/>
+      <c r="G14" s="125"/>
+      <c r="H14" s="125"/>
+      <c r="I14" s="126"/>
+      <c r="J14" s="128"/>
+      <c r="K14" s="129"/>
     </row>
     <row r="15" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A15" s="53"/>
@@ -10201,18 +10319,18 @@
       <c r="D15" s="54"/>
       <c r="E15" s="56">
         <f>SUM(E5:E14)</f>
-        <v>170</v>
+        <v>130</v>
       </c>
       <c r="F15" s="54"/>
       <c r="G15" s="57"/>
       <c r="H15" s="57"/>
       <c r="I15" s="56">
         <f>SUM(I5:I14)</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J15" s="58">
         <f>SUM(J5:J14)</f>
-        <v>0</v>
+        <v>-5.5</v>
       </c>
       <c r="K15" s="57"/>
     </row>
@@ -10326,183 +10444,183 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" s="60" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="126" t="s">
-        <v>83</v>
-      </c>
-      <c r="B1" s="126"/>
-      <c r="C1" s="126"/>
-      <c r="D1" s="126"/>
-      <c r="E1" s="126"/>
-      <c r="F1" s="126"/>
-      <c r="G1" s="126"/>
-      <c r="H1" s="126"/>
-      <c r="I1" s="126"/>
-      <c r="J1" s="126"/>
-      <c r="K1" s="126"/>
+      <c r="A1" s="130" t="s">
+        <v>82</v>
+      </c>
+      <c r="B1" s="130"/>
+      <c r="C1" s="130"/>
+      <c r="D1" s="130"/>
+      <c r="E1" s="130"/>
+      <c r="F1" s="130"/>
+      <c r="G1" s="130"/>
+      <c r="H1" s="130"/>
+      <c r="I1" s="130"/>
+      <c r="J1" s="130"/>
+      <c r="K1" s="130"/>
     </row>
     <row r="2" spans="1:11" hidden="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="D3" s="62" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="21" hidden="1" x14ac:dyDescent="0.25">
       <c r="D4" s="63" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="5" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="D5" s="63" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="6" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="D6" s="63" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="21" hidden="1" x14ac:dyDescent="0.25">
       <c r="D7" s="63" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="8" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="D8" s="63" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="9" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="D9" s="63" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="10" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="D10" s="63" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="11" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="D11" s="63" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="12" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="D12" s="63" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="13" spans="1:11" ht="21" hidden="1" x14ac:dyDescent="0.25">
       <c r="D13" s="63" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="14" spans="1:11" ht="21" hidden="1" x14ac:dyDescent="0.25">
       <c r="D14" s="62" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="15" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="D15" s="63" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="16" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="D16" s="63" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="17" spans="4:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="D17" s="63" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="18" spans="4:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="D18" s="62" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="19" spans="4:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="D19" s="63" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="20" spans="4:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="D20" s="63" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="21" spans="4:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="D21" s="63" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="22" spans="4:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="D22" s="62" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="23" spans="4:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="D23" s="63" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="24" spans="4:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="D24" s="63" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="25" spans="4:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="D25" s="63" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="26" spans="4:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="D26" s="63" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="27" spans="4:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="D27" s="62" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="28" spans="4:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="D28" s="63" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="29" spans="4:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="D29" s="63" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="30" spans="4:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="D30" s="63" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="31" spans="4:4" s="64" customFormat="1" ht="10.199999999999999" hidden="1" x14ac:dyDescent="0.2">
       <c r="D31" s="65" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="32" spans="4:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="D32" s="66" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" ht="22.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D33" s="145" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="33" spans="1:11" ht="22.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D33" s="131" t="s">
-        <v>114</v>
-      </c>
-      <c r="E33" s="131"/>
+      <c r="E33" s="145"/>
     </row>
     <row r="34" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="D34" s="63">
         <v>4290</v>
       </c>
       <c r="E34" s="63" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="35" spans="1:11" ht="21" hidden="1" x14ac:dyDescent="0.25">
@@ -10510,7 +10628,7 @@
         <v>5082</v>
       </c>
       <c r="E35" s="63" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="36" spans="1:11" ht="21" hidden="1" x14ac:dyDescent="0.25">
@@ -10518,7 +10636,7 @@
         <v>4356</v>
       </c>
       <c r="E36" s="63" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="37" spans="1:11" ht="21" hidden="1" x14ac:dyDescent="0.25">
@@ -10526,7 +10644,7 @@
         <v>5929</v>
       </c>
       <c r="E37" s="63" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="38" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
@@ -10534,7 +10652,7 @@
         <v>5005</v>
       </c>
       <c r="E38" s="63" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="39" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
@@ -10542,147 +10660,147 @@
         <v>4225</v>
       </c>
       <c r="E39" s="63" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="40" spans="1:11" ht="8.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="41" spans="1:11" s="60" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="132" t="s">
+      <c r="A41" s="146" t="s">
+        <v>120</v>
+      </c>
+      <c r="B41" s="146"/>
+      <c r="C41" s="146"/>
+      <c r="D41" s="146"/>
+      <c r="E41" s="146"/>
+      <c r="F41" s="146"/>
+      <c r="G41" s="146"/>
+      <c r="H41" s="146"/>
+      <c r="I41" s="146"/>
+      <c r="J41" s="146"/>
+      <c r="K41" s="146"/>
+    </row>
+    <row r="42" spans="1:11" s="60" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="147" t="s">
         <v>121</v>
       </c>
-      <c r="B41" s="132"/>
-      <c r="C41" s="132"/>
-      <c r="D41" s="132"/>
-      <c r="E41" s="132"/>
-      <c r="F41" s="132"/>
-      <c r="G41" s="132"/>
-      <c r="H41" s="132"/>
-      <c r="I41" s="132"/>
-      <c r="J41" s="132"/>
-      <c r="K41" s="132"/>
-    </row>
-    <row r="42" spans="1:11" s="60" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="133" t="s">
+      <c r="B42" s="147"/>
+      <c r="C42" s="147"/>
+      <c r="D42" s="147"/>
+      <c r="E42" s="147"/>
+      <c r="F42" s="147"/>
+      <c r="G42" s="147"/>
+      <c r="H42" s="147"/>
+      <c r="I42" s="147"/>
+      <c r="J42" s="147"/>
+      <c r="K42" s="147"/>
+    </row>
+    <row r="43" spans="1:11" s="60" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="148" t="s">
         <v>122</v>
       </c>
-      <c r="B42" s="133"/>
-      <c r="C42" s="133"/>
-      <c r="D42" s="133"/>
-      <c r="E42" s="133"/>
-      <c r="F42" s="133"/>
-      <c r="G42" s="133"/>
-      <c r="H42" s="133"/>
-      <c r="I42" s="133"/>
-      <c r="J42" s="133"/>
-      <c r="K42" s="133"/>
-    </row>
-    <row r="43" spans="1:11" s="60" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="134" t="s">
+      <c r="B43" s="148"/>
+      <c r="C43" s="148"/>
+      <c r="D43" s="148"/>
+      <c r="E43" s="148"/>
+      <c r="F43" s="148"/>
+      <c r="G43" s="148"/>
+      <c r="H43" s="148"/>
+      <c r="I43" s="148"/>
+      <c r="J43" s="148"/>
+      <c r="K43" s="148"/>
+    </row>
+    <row r="44" spans="1:11" s="60" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="144" t="s">
         <v>123</v>
       </c>
-      <c r="B43" s="134"/>
-      <c r="C43" s="134"/>
-      <c r="D43" s="134"/>
-      <c r="E43" s="134"/>
-      <c r="F43" s="134"/>
-      <c r="G43" s="134"/>
-      <c r="H43" s="134"/>
-      <c r="I43" s="134"/>
-      <c r="J43" s="134"/>
-      <c r="K43" s="134"/>
-    </row>
-    <row r="44" spans="1:11" s="60" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="130" t="s">
-        <v>124</v>
-      </c>
-      <c r="B44" s="130"/>
-      <c r="C44" s="130"/>
-      <c r="D44" s="130"/>
-      <c r="E44" s="130"/>
-      <c r="F44" s="130"/>
-      <c r="G44" s="130"/>
-      <c r="H44" s="130"/>
-      <c r="I44" s="130"/>
-      <c r="J44" s="130"/>
-      <c r="K44" s="130"/>
+      <c r="B44" s="144"/>
+      <c r="C44" s="144"/>
+      <c r="D44" s="144"/>
+      <c r="E44" s="144"/>
+      <c r="F44" s="144"/>
+      <c r="G44" s="144"/>
+      <c r="H44" s="144"/>
+      <c r="I44" s="144"/>
+      <c r="J44" s="144"/>
+      <c r="K44" s="144"/>
     </row>
     <row r="45" spans="1:11" ht="9" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="46" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A46" s="137" t="s">
-        <v>125</v>
-      </c>
-      <c r="B46" s="137"/>
-      <c r="C46" s="137"/>
-      <c r="D46" s="137"/>
-      <c r="E46" s="137"/>
-      <c r="F46" s="137"/>
-      <c r="G46" s="137"/>
-      <c r="H46" s="137"/>
-      <c r="I46" s="137"/>
-      <c r="J46" s="137"/>
-      <c r="K46" s="137"/>
+      <c r="A46" s="151" t="s">
+        <v>124</v>
+      </c>
+      <c r="B46" s="151"/>
+      <c r="C46" s="151"/>
+      <c r="D46" s="151"/>
+      <c r="E46" s="151"/>
+      <c r="F46" s="151"/>
+      <c r="G46" s="151"/>
+      <c r="H46" s="151"/>
+      <c r="I46" s="151"/>
+      <c r="J46" s="151"/>
+      <c r="K46" s="151"/>
     </row>
     <row r="47" spans="1:11" s="69" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="67" t="s">
+        <v>125</v>
+      </c>
+      <c r="B47" s="68"/>
+      <c r="C47" s="152" t="s">
         <v>126</v>
       </c>
-      <c r="B47" s="68"/>
-      <c r="C47" s="138" t="s">
+      <c r="D47" s="152"/>
+      <c r="E47" s="152"/>
+      <c r="F47" s="152"/>
+      <c r="G47" s="152"/>
+      <c r="H47" s="152"/>
+      <c r="I47" s="152"/>
+      <c r="J47" s="152"/>
+      <c r="K47" s="152"/>
+    </row>
+    <row r="48" spans="1:11" s="71" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="153"/>
+      <c r="B48" s="149" t="s">
         <v>127</v>
       </c>
-      <c r="D47" s="138"/>
-      <c r="E47" s="138"/>
-      <c r="F47" s="138"/>
-      <c r="G47" s="138"/>
-      <c r="H47" s="138"/>
-      <c r="I47" s="138"/>
-      <c r="J47" s="138"/>
-      <c r="K47" s="138"/>
-    </row>
-    <row r="48" spans="1:11" s="71" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="139"/>
-      <c r="B48" s="135" t="s">
+      <c r="C48" s="149" t="s">
         <v>128</v>
       </c>
-      <c r="C48" s="135" t="s">
+      <c r="D48" s="149" t="s">
         <v>129</v>
       </c>
-      <c r="D48" s="135" t="s">
+      <c r="E48" s="149" t="s">
+        <v>98</v>
+      </c>
+      <c r="F48" s="149" t="s">
         <v>130</v>
       </c>
-      <c r="E48" s="135" t="s">
-        <v>99</v>
-      </c>
-      <c r="F48" s="135" t="s">
+      <c r="G48" s="149" t="s">
+        <v>102</v>
+      </c>
+      <c r="H48" s="154" t="s">
         <v>131</v>
       </c>
-      <c r="G48" s="135" t="s">
-        <v>103</v>
-      </c>
-      <c r="H48" s="140" t="s">
+      <c r="I48" s="154"/>
+      <c r="J48" s="154"/>
+      <c r="K48" s="154"/>
+    </row>
+    <row r="49" spans="1:11" s="71" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A49" s="153"/>
+      <c r="B49" s="149"/>
+      <c r="C49" s="149"/>
+      <c r="D49" s="149"/>
+      <c r="E49" s="149"/>
+      <c r="F49" s="149"/>
+      <c r="G49" s="149"/>
+      <c r="H49" s="149" t="s">
         <v>132</v>
       </c>
-      <c r="I48" s="140"/>
-      <c r="J48" s="140"/>
-      <c r="K48" s="140"/>
-    </row>
-    <row r="49" spans="1:11" s="71" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="139"/>
-      <c r="B49" s="135"/>
-      <c r="C49" s="135"/>
-      <c r="D49" s="135"/>
-      <c r="E49" s="135"/>
-      <c r="F49" s="135"/>
-      <c r="G49" s="135"/>
-      <c r="H49" s="135" t="s">
+      <c r="I49" s="149"/>
+      <c r="J49" s="70" t="s">
         <v>133</v>
       </c>
-      <c r="I49" s="135"/>
-      <c r="J49" s="70" t="s">
+      <c r="K49" s="70" t="s">
         <v>134</v>
-      </c>
-      <c r="K49" s="70" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="50" spans="1:11" s="71" customFormat="1" ht="40.799999999999997" x14ac:dyDescent="0.25">
@@ -10690,31 +10808,31 @@
         <v>1</v>
       </c>
       <c r="B50" s="73" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C50" s="74">
         <v>46252</v>
       </c>
       <c r="D50" s="75" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E50" s="75" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F50" s="76" t="str">
         <f t="shared" ref="F50:F60" si="0">IF(OR((CODE($D50)*CODE($E50))=$D$36,(CODE($D50)*CODE($E50))=$D$35),$D$15,IF(OR((CODE($D50)*CODE($E50))=$D$34,(CODE($D50)*CODE($E50))=$D$37),$D$16,IF(OR((CODE($D50)*CODE($E50))=$D$38,(CODE($D50)*CODE($E50))=$D$39),$D$17,0)))</f>
         <v>Alta</v>
       </c>
       <c r="G50" s="75" t="s">
-        <v>104</v>
-      </c>
-      <c r="H50" s="136"/>
-      <c r="I50" s="136"/>
+        <v>103</v>
+      </c>
+      <c r="H50" s="150"/>
+      <c r="I50" s="150"/>
       <c r="J50" s="77" t="s">
-        <v>236</v>
+        <v>227</v>
       </c>
       <c r="K50" s="77" t="s">
-        <v>237</v>
+        <v>228</v>
       </c>
     </row>
     <row r="51" spans="1:11" s="71" customFormat="1" ht="51" x14ac:dyDescent="0.25">
@@ -10722,31 +10840,31 @@
         <v>2</v>
       </c>
       <c r="B51" s="73" t="s">
-        <v>238</v>
+        <v>229</v>
       </c>
       <c r="C51" s="74">
         <v>46252</v>
       </c>
       <c r="D51" s="75" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E51" s="75" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F51" s="76" t="str">
         <f t="shared" si="0"/>
         <v>Alta</v>
       </c>
       <c r="G51" s="75" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="H51" s="78"/>
       <c r="I51" s="79"/>
       <c r="J51" s="77" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="K51" s="77" t="s">
-        <v>240</v>
+        <v>231</v>
       </c>
     </row>
     <row r="52" spans="1:11" s="71" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -10872,8 +10990,8 @@
         <v>#VALUE!</v>
       </c>
       <c r="G59" s="75"/>
-      <c r="H59" s="136"/>
-      <c r="I59" s="136"/>
+      <c r="H59" s="150"/>
+      <c r="I59" s="150"/>
       <c r="J59" s="77"/>
       <c r="K59" s="77"/>
     </row>
@@ -10888,8 +11006,8 @@
         <v>#VALUE!</v>
       </c>
       <c r="G60" s="75"/>
-      <c r="H60" s="136"/>
-      <c r="I60" s="136"/>
+      <c r="H60" s="150"/>
+      <c r="I60" s="150"/>
       <c r="J60" s="77"/>
       <c r="K60" s="77"/>
     </row>
@@ -10972,167 +11090,167 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:23" s="60" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="143" t="s">
+      <c r="A1" s="157" t="s">
+        <v>136</v>
+      </c>
+      <c r="B1" s="157"/>
+      <c r="C1" s="157"/>
+      <c r="D1" s="157"/>
+      <c r="E1" s="157"/>
+      <c r="F1" s="157"/>
+      <c r="G1" s="157"/>
+      <c r="H1" s="157"/>
+      <c r="I1" s="157"/>
+      <c r="J1" s="157"/>
+      <c r="K1" s="157"/>
+      <c r="L1" s="157"/>
+      <c r="M1" s="157"/>
+      <c r="N1" s="157"/>
+    </row>
+    <row r="2" spans="1:23" s="80" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="158" t="s">
+        <v>120</v>
+      </c>
+      <c r="B2" s="158"/>
+      <c r="C2" s="158"/>
+      <c r="D2" s="158"/>
+      <c r="E2" s="158"/>
+      <c r="F2" s="158"/>
+      <c r="G2" s="158"/>
+      <c r="H2" s="158"/>
+      <c r="I2" s="158"/>
+      <c r="J2" s="158"/>
+      <c r="K2" s="158"/>
+      <c r="L2" s="158"/>
+      <c r="M2" s="158"/>
+      <c r="N2" s="158"/>
+    </row>
+    <row r="3" spans="1:23" s="80" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="159" t="s">
         <v>137</v>
       </c>
-      <c r="B1" s="143"/>
-      <c r="C1" s="143"/>
-      <c r="D1" s="143"/>
-      <c r="E1" s="143"/>
-      <c r="F1" s="143"/>
-      <c r="G1" s="143"/>
-      <c r="H1" s="143"/>
-      <c r="I1" s="143"/>
-      <c r="J1" s="143"/>
-      <c r="K1" s="143"/>
-      <c r="L1" s="143"/>
-      <c r="M1" s="143"/>
-      <c r="N1" s="143"/>
-    </row>
-    <row r="2" spans="1:23" s="80" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="144" t="s">
-        <v>121</v>
-      </c>
-      <c r="B2" s="144"/>
-      <c r="C2" s="144"/>
-      <c r="D2" s="144"/>
-      <c r="E2" s="144"/>
-      <c r="F2" s="144"/>
-      <c r="G2" s="144"/>
-      <c r="H2" s="144"/>
-      <c r="I2" s="144"/>
-      <c r="J2" s="144"/>
-      <c r="K2" s="144"/>
-      <c r="L2" s="144"/>
-      <c r="M2" s="144"/>
-      <c r="N2" s="144"/>
-    </row>
-    <row r="3" spans="1:23" s="80" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="145" t="s">
+      <c r="B3" s="159"/>
+      <c r="C3" s="159"/>
+      <c r="D3" s="159"/>
+      <c r="E3" s="159"/>
+      <c r="F3" s="159"/>
+      <c r="G3" s="159"/>
+      <c r="H3" s="159"/>
+      <c r="I3" s="159"/>
+      <c r="J3" s="159"/>
+      <c r="K3" s="159"/>
+      <c r="L3" s="159"/>
+      <c r="M3" s="159"/>
+      <c r="N3" s="159"/>
+    </row>
+    <row r="4" spans="1:23" s="80" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="160" t="s">
         <v>138</v>
       </c>
-      <c r="B3" s="145"/>
-      <c r="C3" s="145"/>
-      <c r="D3" s="145"/>
-      <c r="E3" s="145"/>
-      <c r="F3" s="145"/>
-      <c r="G3" s="145"/>
-      <c r="H3" s="145"/>
-      <c r="I3" s="145"/>
-      <c r="J3" s="145"/>
-      <c r="K3" s="145"/>
-      <c r="L3" s="145"/>
-      <c r="M3" s="145"/>
-      <c r="N3" s="145"/>
-    </row>
-    <row r="4" spans="1:23" s="80" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="146" t="s">
+      <c r="B4" s="160"/>
+      <c r="C4" s="160"/>
+      <c r="D4" s="160"/>
+      <c r="E4" s="160"/>
+      <c r="F4" s="160"/>
+      <c r="G4" s="160"/>
+      <c r="H4" s="160"/>
+      <c r="I4" s="160"/>
+      <c r="J4" s="160"/>
+      <c r="K4" s="160"/>
+      <c r="L4" s="160"/>
+      <c r="M4" s="160"/>
+      <c r="N4" s="160"/>
+    </row>
+    <row r="5" spans="1:23" s="80" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="161" t="s">
         <v>139</v>
       </c>
-      <c r="B4" s="146"/>
-      <c r="C4" s="146"/>
-      <c r="D4" s="146"/>
-      <c r="E4" s="146"/>
-      <c r="F4" s="146"/>
-      <c r="G4" s="146"/>
-      <c r="H4" s="146"/>
-      <c r="I4" s="146"/>
-      <c r="J4" s="146"/>
-      <c r="K4" s="146"/>
-      <c r="L4" s="146"/>
-      <c r="M4" s="146"/>
-      <c r="N4" s="146"/>
-    </row>
-    <row r="5" spans="1:23" s="80" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="147" t="s">
-        <v>140</v>
-      </c>
-      <c r="B5" s="147"/>
-      <c r="C5" s="147"/>
-      <c r="D5" s="147"/>
-      <c r="E5" s="147"/>
-      <c r="F5" s="147"/>
-      <c r="G5" s="147"/>
-      <c r="H5" s="147"/>
-      <c r="I5" s="147"/>
-      <c r="J5" s="147"/>
-      <c r="K5" s="147"/>
-      <c r="L5" s="147"/>
-      <c r="M5" s="147"/>
-      <c r="N5" s="147"/>
+      <c r="B5" s="161"/>
+      <c r="C5" s="161"/>
+      <c r="D5" s="161"/>
+      <c r="E5" s="161"/>
+      <c r="F5" s="161"/>
+      <c r="G5" s="161"/>
+      <c r="H5" s="161"/>
+      <c r="I5" s="161"/>
+      <c r="J5" s="161"/>
+      <c r="K5" s="161"/>
+      <c r="L5" s="161"/>
+      <c r="M5" s="161"/>
+      <c r="N5" s="161"/>
     </row>
     <row r="6" spans="1:23" s="4" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="7" spans="1:23" s="4" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="141" t="s">
+      <c r="A7" s="155" t="s">
+        <v>140</v>
+      </c>
+      <c r="B7" s="155"/>
+      <c r="D7" s="155" t="s">
         <v>141</v>
       </c>
-      <c r="B7" s="141"/>
-      <c r="D7" s="141" t="s">
+      <c r="E7" s="155"/>
+      <c r="G7" s="155" t="s">
         <v>142</v>
       </c>
-      <c r="E7" s="141"/>
-      <c r="G7" s="141" t="s">
+      <c r="H7" s="155"/>
+      <c r="I7" s="155"/>
+      <c r="J7" s="155"/>
+      <c r="K7" s="155"/>
+      <c r="M7" s="155" t="s">
         <v>143</v>
       </c>
-      <c r="H7" s="141"/>
-      <c r="I7" s="141"/>
-      <c r="J7" s="141"/>
-      <c r="K7" s="141"/>
-      <c r="M7" s="141" t="s">
-        <v>144</v>
-      </c>
-      <c r="N7" s="141"/>
+      <c r="N7" s="155"/>
     </row>
     <row r="8" spans="1:23" s="4" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="83" t="s">
+        <v>144</v>
+      </c>
+      <c r="B8" s="84" t="s">
         <v>145</v>
       </c>
-      <c r="B8" s="84" t="s">
+      <c r="D8" s="83" t="s">
         <v>146</v>
       </c>
-      <c r="D8" s="83" t="s">
+      <c r="E8" s="84" t="s">
+        <v>145</v>
+      </c>
+      <c r="G8" s="83" t="s">
         <v>147</v>
       </c>
-      <c r="E8" s="84" t="s">
-        <v>146</v>
-      </c>
-      <c r="G8" s="83" t="s">
+      <c r="H8" s="83" t="s">
         <v>148</v>
       </c>
-      <c r="H8" s="83" t="s">
+      <c r="I8" s="83" t="s">
+        <v>96</v>
+      </c>
+      <c r="J8" s="84" t="s">
         <v>149</v>
       </c>
-      <c r="I8" s="83" t="s">
-        <v>97</v>
-      </c>
-      <c r="J8" s="84" t="s">
+      <c r="K8" s="84" t="s">
         <v>150</v>
       </c>
-      <c r="K8" s="84" t="s">
+      <c r="M8" s="84" t="s">
         <v>151</v>
       </c>
-      <c r="M8" s="84" t="s">
+      <c r="N8" s="84" t="s">
         <v>152</v>
-      </c>
-      <c r="N8" s="84" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="9" spans="1:23" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.25">
       <c r="A9" s="81" t="s">
+        <v>153</v>
+      </c>
+      <c r="B9" s="82" t="s">
+        <v>148</v>
+      </c>
+      <c r="D9" s="81" t="s">
         <v>154</v>
       </c>
-      <c r="B9" s="82" t="s">
-        <v>149</v>
-      </c>
-      <c r="D9" s="81" t="s">
+      <c r="E9" s="82" t="s">
+        <v>148</v>
+      </c>
+      <c r="G9" s="83" t="s">
         <v>155</v>
-      </c>
-      <c r="E9" s="82" t="s">
-        <v>149</v>
-      </c>
-      <c r="G9" s="83" t="s">
-        <v>156</v>
       </c>
       <c r="H9" s="81">
         <v>2</v>
@@ -11148,21 +11266,21 @@
         <v>8</v>
       </c>
       <c r="M9" s="85" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="N9" s="86"/>
     </row>
     <row r="10" spans="1:23" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.25">
       <c r="A10" s="81" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B10" s="82" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D10" s="81"/>
       <c r="E10" s="82"/>
       <c r="G10" s="83" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="H10" s="81"/>
       <c r="I10" s="81"/>
@@ -11172,7 +11290,7 @@
         <v>0</v>
       </c>
       <c r="M10" s="85" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="N10" s="86"/>
     </row>
@@ -11181,15 +11299,15 @@
       <c r="B11" s="82"/>
       <c r="D11" s="81"/>
       <c r="E11" s="82"/>
-      <c r="G11" s="141" t="s">
+      <c r="G11" s="155" t="s">
+        <v>160</v>
+      </c>
+      <c r="H11" s="155"/>
+      <c r="I11" s="155"/>
+      <c r="J11" s="155"/>
+      <c r="K11" s="155"/>
+      <c r="M11" s="85" t="s">
         <v>161</v>
-      </c>
-      <c r="H11" s="141"/>
-      <c r="I11" s="141"/>
-      <c r="J11" s="141"/>
-      <c r="K11" s="141"/>
-      <c r="M11" s="85" t="s">
-        <v>162</v>
       </c>
       <c r="N11" s="86"/>
     </row>
@@ -11199,22 +11317,22 @@
       <c r="D12" s="81"/>
       <c r="E12" s="82"/>
       <c r="G12" s="83" t="s">
+        <v>147</v>
+      </c>
+      <c r="H12" s="83" t="s">
         <v>148</v>
       </c>
-      <c r="H12" s="83" t="s">
+      <c r="I12" s="83" t="s">
+        <v>96</v>
+      </c>
+      <c r="J12" s="84" t="s">
         <v>149</v>
       </c>
-      <c r="I12" s="83" t="s">
-        <v>97</v>
-      </c>
-      <c r="J12" s="84" t="s">
+      <c r="K12" s="84" t="s">
         <v>150</v>
       </c>
-      <c r="K12" s="84" t="s">
-        <v>151</v>
-      </c>
       <c r="M12" s="85" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="N12" s="86"/>
     </row>
@@ -11224,7 +11342,7 @@
       <c r="D13" s="81"/>
       <c r="E13" s="82"/>
       <c r="G13" s="83" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="H13" s="81">
         <v>1</v>
@@ -11236,11 +11354,11 @@
         <v>3</v>
       </c>
       <c r="M13" s="85" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="N13" s="86"/>
       <c r="W13" s="4" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="14" spans="1:23" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.25">
@@ -11249,7 +11367,7 @@
       <c r="D14" s="81"/>
       <c r="E14" s="82"/>
       <c r="G14" s="83" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="H14" s="81"/>
       <c r="I14" s="81"/>
@@ -11259,7 +11377,7 @@
         <v>0</v>
       </c>
       <c r="M14" s="85" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="N14" s="86"/>
     </row>
@@ -11269,7 +11387,7 @@
       <c r="D15" s="81"/>
       <c r="E15" s="82"/>
       <c r="G15" s="83" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="H15" s="81">
         <v>1</v>
@@ -11281,7 +11399,7 @@
         <v>3</v>
       </c>
       <c r="M15" s="85" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="N15" s="86"/>
     </row>
@@ -11290,18 +11408,18 @@
       <c r="B16" s="82"/>
       <c r="D16" s="81"/>
       <c r="E16" s="82"/>
-      <c r="G16" s="142" t="s">
-        <v>171</v>
-      </c>
-      <c r="H16" s="142"/>
-      <c r="I16" s="142"/>
-      <c r="J16" s="142"/>
+      <c r="G16" s="156" t="s">
+        <v>170</v>
+      </c>
+      <c r="H16" s="156"/>
+      <c r="I16" s="156"/>
+      <c r="J16" s="156"/>
       <c r="K16" s="87">
         <f>SUM(K9,K10,K13,K14,K15)</f>
         <v>14</v>
       </c>
       <c r="M16" s="85" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="N16" s="86"/>
     </row>
@@ -11311,7 +11429,7 @@
       <c r="D17" s="81"/>
       <c r="E17" s="82"/>
       <c r="M17" s="85" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="N17" s="86"/>
     </row>
@@ -11321,7 +11439,7 @@
       <c r="D18" s="81"/>
       <c r="E18" s="82"/>
       <c r="M18" s="85" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="N18" s="86"/>
     </row>
@@ -11331,7 +11449,7 @@
       <c r="D19" s="81"/>
       <c r="E19" s="82"/>
       <c r="M19" s="85" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="N19" s="86"/>
     </row>
@@ -11341,25 +11459,25 @@
       <c r="D20" s="81"/>
       <c r="E20" s="82"/>
       <c r="M20" s="85" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="N20" s="86"/>
     </row>
     <row r="21" spans="1:14" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.25">
       <c r="M21" s="85" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="N21" s="86"/>
     </row>
     <row r="22" spans="1:14" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.25">
       <c r="M22" s="85" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="N22" s="86"/>
     </row>
     <row r="23" spans="1:14" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.25">
       <c r="M23" s="88" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="N23" s="89">
         <f>SUM(N9:N22)</f>
@@ -11368,7 +11486,7 @@
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.3">
       <c r="M24" s="88" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="N24" s="87">
         <f>(N23*0.01)+0.65</f>
@@ -11377,7 +11495,7 @@
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.3">
       <c r="M25" s="88" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="N25" s="90">
         <f>K16*N24</f>
@@ -11386,7 +11504,7 @@
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.3">
       <c r="M26" s="88" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="N26" s="91">
         <v>19</v>
@@ -11394,7 +11512,7 @@
     </row>
     <row r="27" spans="1:14" ht="21" x14ac:dyDescent="0.3">
       <c r="M27" s="92" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="N27" s="93">
         <f>N25*N26</f>
@@ -11455,118 +11573,118 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="21" x14ac:dyDescent="0.4">
-      <c r="A1" s="143" t="s">
-        <v>44</v>
-      </c>
-      <c r="B1" s="143"/>
-      <c r="C1" s="143"/>
-      <c r="D1" s="143"/>
-      <c r="E1" s="143"/>
-      <c r="F1" s="143"/>
-      <c r="G1" s="143"/>
-      <c r="H1" s="143"/>
-      <c r="I1" s="143"/>
-      <c r="J1" s="143"/>
-      <c r="K1" s="143"/>
-      <c r="L1" s="143"/>
-      <c r="M1" s="143"/>
-      <c r="N1" s="143"/>
+      <c r="A1" s="157" t="s">
+        <v>43</v>
+      </c>
+      <c r="B1" s="157"/>
+      <c r="C1" s="157"/>
+      <c r="D1" s="157"/>
+      <c r="E1" s="157"/>
+      <c r="F1" s="157"/>
+      <c r="G1" s="157"/>
+      <c r="H1" s="157"/>
+      <c r="I1" s="157"/>
+      <c r="J1" s="157"/>
+      <c r="K1" s="157"/>
+      <c r="L1" s="157"/>
+      <c r="M1" s="157"/>
+      <c r="N1" s="157"/>
     </row>
     <row r="2" spans="1:14" ht="7.5" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="3" spans="1:14" ht="18" x14ac:dyDescent="0.35">
-      <c r="A3" s="149" t="s">
-        <v>45</v>
-      </c>
-      <c r="B3" s="149"/>
-      <c r="C3" s="149"/>
-      <c r="E3" s="149" t="s">
-        <v>184</v>
-      </c>
-      <c r="F3" s="149"/>
-      <c r="G3" s="149"/>
-      <c r="H3" s="149"/>
-      <c r="I3" s="149"/>
-      <c r="J3" s="149"/>
-      <c r="K3" s="149"/>
-      <c r="L3" s="149"/>
-      <c r="M3" s="149"/>
-      <c r="N3" s="149"/>
+      <c r="A3" s="163" t="s">
+        <v>44</v>
+      </c>
+      <c r="B3" s="163"/>
+      <c r="C3" s="163"/>
+      <c r="E3" s="163" t="s">
+        <v>183</v>
+      </c>
+      <c r="F3" s="163"/>
+      <c r="G3" s="163"/>
+      <c r="H3" s="163"/>
+      <c r="I3" s="163"/>
+      <c r="J3" s="163"/>
+      <c r="K3" s="163"/>
+      <c r="L3" s="163"/>
+      <c r="M3" s="163"/>
+      <c r="N3" s="163"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" s="94" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B4" s="95">
         <f>'#Estimativa-APF#'!$N$27</f>
         <v>172.9</v>
       </c>
       <c r="C4" s="29" t="s">
-        <v>47</v>
-      </c>
-      <c r="E4" s="150" t="s">
-        <v>186</v>
-      </c>
-      <c r="F4" s="148" t="s">
+        <v>46</v>
+      </c>
+      <c r="E4" s="164" t="s">
+        <v>185</v>
+      </c>
+      <c r="F4" s="162" t="s">
         <v>16</v>
       </c>
-      <c r="G4" s="148"/>
-      <c r="H4" s="148" t="s">
+      <c r="G4" s="162"/>
+      <c r="H4" s="162" t="s">
         <v>30</v>
       </c>
-      <c r="I4" s="148"/>
-      <c r="J4" s="148" t="s">
+      <c r="I4" s="162"/>
+      <c r="J4" s="162" t="s">
+        <v>35</v>
+      </c>
+      <c r="K4" s="162"/>
+      <c r="L4" s="162" t="s">
         <v>36</v>
       </c>
-      <c r="K4" s="148"/>
-      <c r="L4" s="148" t="s">
-        <v>37</v>
-      </c>
-      <c r="M4" s="148"/>
+      <c r="M4" s="162"/>
       <c r="N4" s="96"/>
     </row>
     <row r="5" spans="1:14" ht="18" x14ac:dyDescent="0.35">
       <c r="A5" s="27" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B5" s="28">
         <v>0</v>
       </c>
       <c r="C5" s="37" t="s">
+        <v>186</v>
+      </c>
+      <c r="E5" s="164"/>
+      <c r="F5" s="162" t="s">
+        <v>17</v>
+      </c>
+      <c r="G5" s="162"/>
+      <c r="H5" s="162" t="s">
+        <v>17</v>
+      </c>
+      <c r="I5" s="162"/>
+      <c r="J5" s="162" t="s">
+        <v>17</v>
+      </c>
+      <c r="K5" s="162"/>
+      <c r="L5" s="162" t="s">
+        <v>17</v>
+      </c>
+      <c r="M5" s="162"/>
+      <c r="N5" s="40" t="s">
         <v>187</v>
-      </c>
-      <c r="E5" s="150"/>
-      <c r="F5" s="148" t="s">
-        <v>17</v>
-      </c>
-      <c r="G5" s="148"/>
-      <c r="H5" s="148" t="s">
-        <v>17</v>
-      </c>
-      <c r="I5" s="148"/>
-      <c r="J5" s="148" t="s">
-        <v>17</v>
-      </c>
-      <c r="K5" s="148"/>
-      <c r="L5" s="148" t="s">
-        <v>17</v>
-      </c>
-      <c r="M5" s="148"/>
-      <c r="N5" s="40" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6" s="97" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B6" s="98">
         <f>B4+(B4*B5)</f>
         <v>172.9</v>
       </c>
       <c r="C6" s="37" t="s">
-        <v>47</v>
-      </c>
-      <c r="E6" s="150"/>
+        <v>46</v>
+      </c>
+      <c r="E6" s="164"/>
       <c r="F6" s="99">
         <f>B6*G6</f>
         <v>8.6450000000000014</v>
@@ -11599,14 +11717,14 @@
     </row>
     <row r="7" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A7" s="29" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B7" s="30">
         <v>1</v>
       </c>
       <c r="C7" s="29"/>
       <c r="E7" s="101" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F7" s="99">
         <f>F6*G7</f>
@@ -11643,16 +11761,16 @@
     </row>
     <row r="8" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A8" s="29" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B8" s="30">
         <v>40</v>
       </c>
       <c r="C8" s="29" t="s">
+        <v>192</v>
+      </c>
+      <c r="E8" s="101" t="s">
         <v>193</v>
-      </c>
-      <c r="E8" s="101" t="s">
-        <v>194</v>
       </c>
       <c r="F8" s="99">
         <f>F6*G8</f>
@@ -11689,16 +11807,16 @@
     </row>
     <row r="9" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A9" s="29" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B9" s="30">
         <v>2</v>
       </c>
       <c r="C9" s="29" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E9" s="101" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="F9" s="99">
         <f>F6*G9</f>
@@ -11735,17 +11853,17 @@
     </row>
     <row r="10" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A10" s="103" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B10" s="104">
         <f>(B7*B8)*B9</f>
         <v>80</v>
       </c>
       <c r="C10" s="103" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E10" s="101" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="F10" s="99">
         <f>F6*G10</f>
@@ -11782,17 +11900,17 @@
     </row>
     <row r="11" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A11" s="94" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B11" s="105">
         <f>B6/B10*2</f>
         <v>4.3224999999999998</v>
       </c>
       <c r="C11" s="94" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E11" s="101" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="F11" s="99">
         <f>F6*G11</f>
@@ -11829,17 +11947,17 @@
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12" s="94" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B12" s="105">
         <f>B11/4</f>
         <v>1.0806249999999999</v>
       </c>
       <c r="C12" s="94" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E12" s="106" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="F12" s="107">
         <f t="shared" ref="F12:M12" si="0">SUM(F7:F11)</f>
@@ -11877,17 +11995,17 @@
     </row>
     <row r="13" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A13" s="103" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B13" s="109">
         <f>B11/B9</f>
         <v>2.1612499999999999</v>
       </c>
       <c r="C13" s="103" t="s">
+        <v>203</v>
+      </c>
+      <c r="E13" s="101" t="s">
         <v>204</v>
-      </c>
-      <c r="E13" s="101" t="s">
-        <v>205</v>
       </c>
       <c r="F13" s="99">
         <f>F6*G13</f>
@@ -11924,7 +12042,7 @@
     </row>
     <row r="14" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="E14" s="101" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="F14" s="99">
         <f>F6*G14</f>
@@ -11961,7 +12079,7 @@
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.3">
       <c r="E15" s="106" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="F15" s="107">
         <f t="shared" ref="F15:M15" si="1">SUM(F13:F14)</f>
@@ -11998,13 +12116,13 @@
       <c r="N15" s="106"/>
     </row>
     <row r="16" spans="1:14" ht="18" x14ac:dyDescent="0.35">
-      <c r="A16" s="149" t="s">
-        <v>61</v>
-      </c>
-      <c r="B16" s="149"/>
-      <c r="C16" s="149"/>
+      <c r="A16" s="163" t="s">
+        <v>60</v>
+      </c>
+      <c r="B16" s="163"/>
+      <c r="C16" s="163"/>
       <c r="E16" s="40" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="F16" s="110">
         <f t="shared" ref="F16:M16" si="2">F12+F15</f>
@@ -12045,7 +12163,7 @@
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A17" s="29" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B17" s="113">
         <v>20</v>
@@ -12055,7 +12173,7 @@
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A18" s="29" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B18" s="38">
         <f>B6*B17</f>
@@ -12067,7 +12185,7 @@
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A19" s="29" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B19" s="28">
         <v>0</v>
@@ -12077,7 +12195,7 @@
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A20" s="29" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B20" s="39">
         <f>B18*B19</f>
@@ -12089,7 +12207,7 @@
     </row>
     <row r="21" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A21" s="25" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B21" s="114">
         <f>B18+B20</f>
@@ -12100,7 +12218,7 @@
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A22" s="29" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B22" s="28">
         <v>0.2</v>
@@ -12110,7 +12228,7 @@
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A23" s="29" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B23" s="42">
         <f>B21*B22</f>
@@ -12120,7 +12238,7 @@
     </row>
     <row r="24" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A24" s="25" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B24" s="114">
         <f>B21+B23</f>

</xml_diff>

<commit_message>
Mudando estado da entrega 1 para Entregue
</commit_message>
<xml_diff>
--- a/6.Gerenciamento de Projeto/BRA - Planejamento e Controle do Projeto.xlsx
+++ b/6.Gerenciamento de Projeto/BRA - Planejamento e Controle do Projeto.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\fabioas\Development\bra-brasileirao_analyst\6.Gerenciamento de Projeto\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51661E92-8239-487E-B887-1507DF87717E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{901D9FD3-C3D1-423C-9CDD-B31180BC1C80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-19310" yWindow="-110" windowWidth="19420" windowHeight="11020" activeTab="3" xr2:uid="{31237A52-FFD1-4E1D-B5BB-391D11929C61}"/>
   </bookViews>
@@ -5552,9 +5552,6 @@
     <t>Release-1.0.0</t>
   </si>
   <si>
-    <t>Em execução</t>
-  </si>
-  <si>
     <t>Extrair dados dos clubes e dos atletas</t>
   </si>
   <si>
@@ -5772,6 +5769,9 @@
   </si>
   <si>
     <t>UC 05, UC 01 e UC 02, Guia de Implantação, Modelo de Implantação, Manual de Suporte e Treinamento e sistema em produção</t>
+  </si>
+  <si>
+    <t>Entregue</t>
   </si>
 </sst>
 </file>
@@ -6749,21 +6749,6 @@
     <xf numFmtId="164" fontId="20" fillId="5" borderId="7" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="28" fillId="12" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="29" fillId="13" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="29" fillId="10" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="28" fillId="3" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="28" fillId="14" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="164" fontId="29" fillId="15" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -6777,6 +6762,21 @@
     <xf numFmtId="0" fontId="0" fillId="15" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="29" fillId="15" borderId="4" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="28" fillId="12" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="29" fillId="13" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="29" fillId="10" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="28" fillId="3" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="28" fillId="14" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="16" fillId="13" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -9034,7 +9034,7 @@
         <v>3</v>
       </c>
       <c r="G7" s="12" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="H7" s="15">
         <v>8</v>
@@ -9250,7 +9250,7 @@
         <v>30</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="D15" s="13">
         <v>8</v>
@@ -9271,7 +9271,7 @@
         <v>30</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="D16" s="13">
         <v>0.5</v>
@@ -9292,7 +9292,7 @@
         <v>30</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="D17" s="13">
         <v>1</v>
@@ -9334,7 +9334,7 @@
         <v>30</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="D19" s="13">
         <v>8</v>
@@ -9353,7 +9353,7 @@
         <v>30</v>
       </c>
       <c r="C20" s="12" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="D20" s="13">
         <v>2</v>
@@ -9372,7 +9372,7 @@
         <v>30</v>
       </c>
       <c r="C21" s="18" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="D21" s="13">
         <v>1</v>
@@ -9449,7 +9449,7 @@
         <v>35</v>
       </c>
       <c r="C26" s="12" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="D26" s="13">
         <v>1</v>
@@ -9463,7 +9463,7 @@
         <v>35</v>
       </c>
       <c r="C27" s="12" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="D27" s="13">
         <v>20</v>
@@ -9477,7 +9477,7 @@
         <v>35</v>
       </c>
       <c r="C28" s="12" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="D28" s="13">
         <v>1</v>
@@ -9491,7 +9491,7 @@
         <v>35</v>
       </c>
       <c r="C29" s="12" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="D29" s="13">
         <v>20</v>
@@ -9505,7 +9505,7 @@
         <v>35</v>
       </c>
       <c r="C30" s="12" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="D30" s="13">
         <v>1</v>
@@ -9519,7 +9519,7 @@
         <v>35</v>
       </c>
       <c r="C31" s="12" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="D31" s="13">
         <v>8</v>
@@ -9561,7 +9561,7 @@
         <v>35</v>
       </c>
       <c r="C34" s="12" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="D34" s="13">
         <v>2</v>
@@ -9575,7 +9575,7 @@
         <v>35</v>
       </c>
       <c r="C35" s="12" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="D35" s="13">
         <v>5</v>
@@ -10117,7 +10117,7 @@
         <v>1</v>
       </c>
       <c r="B5" s="116" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C5" s="117">
         <v>46252</v>
@@ -10129,19 +10129,19 @@
         <v>10.5</v>
       </c>
       <c r="F5" s="119" t="s">
-        <v>233</v>
+        <v>252</v>
       </c>
       <c r="G5" s="117">
         <v>46252</v>
       </c>
       <c r="H5" s="117">
-        <v>46259</v>
+        <v>46266</v>
       </c>
       <c r="I5" s="118">
-        <v>5</v>
+        <v>10.5</v>
       </c>
       <c r="J5" s="120">
-        <v>-5.5</v>
+        <v>0</v>
       </c>
       <c r="K5" s="121" t="s">
         <v>232</v>
@@ -10152,7 +10152,7 @@
         <v>2</v>
       </c>
       <c r="B6" s="116" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="C6" s="117">
         <v>46273</v>
@@ -10177,7 +10177,7 @@
         <v>3</v>
       </c>
       <c r="B7" s="116" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="C7" s="117">
         <v>46294</v>
@@ -10202,7 +10202,7 @@
         <v>4</v>
       </c>
       <c r="B8" s="124" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="C8" s="125">
         <v>46315</v>
@@ -10326,11 +10326,11 @@
       <c r="H15" s="57"/>
       <c r="I15" s="56">
         <f>SUM(I5:I14)</f>
-        <v>5</v>
+        <v>10.5</v>
       </c>
       <c r="J15" s="58">
         <f>SUM(J5:J14)</f>
-        <v>-5.5</v>
+        <v>0</v>
       </c>
       <c r="K15" s="57"/>
     </row>
@@ -10610,10 +10610,10 @@
       </c>
     </row>
     <row r="33" spans="1:11" ht="22.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D33" s="145" t="s">
+      <c r="D33" s="151" t="s">
         <v>113</v>
       </c>
-      <c r="E33" s="145"/>
+      <c r="E33" s="151"/>
     </row>
     <row r="34" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="D34" s="63">
@@ -10665,137 +10665,137 @@
     </row>
     <row r="40" spans="1:11" ht="8.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="41" spans="1:11" s="60" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="146" t="s">
+      <c r="A41" s="152" t="s">
         <v>120</v>
       </c>
-      <c r="B41" s="146"/>
-      <c r="C41" s="146"/>
-      <c r="D41" s="146"/>
-      <c r="E41" s="146"/>
-      <c r="F41" s="146"/>
-      <c r="G41" s="146"/>
-      <c r="H41" s="146"/>
-      <c r="I41" s="146"/>
-      <c r="J41" s="146"/>
-      <c r="K41" s="146"/>
+      <c r="B41" s="152"/>
+      <c r="C41" s="152"/>
+      <c r="D41" s="152"/>
+      <c r="E41" s="152"/>
+      <c r="F41" s="152"/>
+      <c r="G41" s="152"/>
+      <c r="H41" s="152"/>
+      <c r="I41" s="152"/>
+      <c r="J41" s="152"/>
+      <c r="K41" s="152"/>
     </row>
     <row r="42" spans="1:11" s="60" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="147" t="s">
+      <c r="A42" s="153" t="s">
         <v>121</v>
       </c>
-      <c r="B42" s="147"/>
-      <c r="C42" s="147"/>
-      <c r="D42" s="147"/>
-      <c r="E42" s="147"/>
-      <c r="F42" s="147"/>
-      <c r="G42" s="147"/>
-      <c r="H42" s="147"/>
-      <c r="I42" s="147"/>
-      <c r="J42" s="147"/>
-      <c r="K42" s="147"/>
+      <c r="B42" s="153"/>
+      <c r="C42" s="153"/>
+      <c r="D42" s="153"/>
+      <c r="E42" s="153"/>
+      <c r="F42" s="153"/>
+      <c r="G42" s="153"/>
+      <c r="H42" s="153"/>
+      <c r="I42" s="153"/>
+      <c r="J42" s="153"/>
+      <c r="K42" s="153"/>
     </row>
     <row r="43" spans="1:11" s="60" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="148" t="s">
+      <c r="A43" s="154" t="s">
         <v>122</v>
       </c>
-      <c r="B43" s="148"/>
-      <c r="C43" s="148"/>
-      <c r="D43" s="148"/>
-      <c r="E43" s="148"/>
-      <c r="F43" s="148"/>
-      <c r="G43" s="148"/>
-      <c r="H43" s="148"/>
-      <c r="I43" s="148"/>
-      <c r="J43" s="148"/>
-      <c r="K43" s="148"/>
+      <c r="B43" s="154"/>
+      <c r="C43" s="154"/>
+      <c r="D43" s="154"/>
+      <c r="E43" s="154"/>
+      <c r="F43" s="154"/>
+      <c r="G43" s="154"/>
+      <c r="H43" s="154"/>
+      <c r="I43" s="154"/>
+      <c r="J43" s="154"/>
+      <c r="K43" s="154"/>
     </row>
     <row r="44" spans="1:11" s="60" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="144" t="s">
+      <c r="A44" s="150" t="s">
         <v>123</v>
       </c>
-      <c r="B44" s="144"/>
-      <c r="C44" s="144"/>
-      <c r="D44" s="144"/>
-      <c r="E44" s="144"/>
-      <c r="F44" s="144"/>
-      <c r="G44" s="144"/>
-      <c r="H44" s="144"/>
-      <c r="I44" s="144"/>
-      <c r="J44" s="144"/>
-      <c r="K44" s="144"/>
+      <c r="B44" s="150"/>
+      <c r="C44" s="150"/>
+      <c r="D44" s="150"/>
+      <c r="E44" s="150"/>
+      <c r="F44" s="150"/>
+      <c r="G44" s="150"/>
+      <c r="H44" s="150"/>
+      <c r="I44" s="150"/>
+      <c r="J44" s="150"/>
+      <c r="K44" s="150"/>
     </row>
     <row r="45" spans="1:11" ht="9" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="46" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A46" s="151" t="s">
+      <c r="A46" s="146" t="s">
         <v>124</v>
       </c>
-      <c r="B46" s="151"/>
-      <c r="C46" s="151"/>
-      <c r="D46" s="151"/>
-      <c r="E46" s="151"/>
-      <c r="F46" s="151"/>
-      <c r="G46" s="151"/>
-      <c r="H46" s="151"/>
-      <c r="I46" s="151"/>
-      <c r="J46" s="151"/>
-      <c r="K46" s="151"/>
+      <c r="B46" s="146"/>
+      <c r="C46" s="146"/>
+      <c r="D46" s="146"/>
+      <c r="E46" s="146"/>
+      <c r="F46" s="146"/>
+      <c r="G46" s="146"/>
+      <c r="H46" s="146"/>
+      <c r="I46" s="146"/>
+      <c r="J46" s="146"/>
+      <c r="K46" s="146"/>
     </row>
     <row r="47" spans="1:11" s="69" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="67" t="s">
         <v>125</v>
       </c>
       <c r="B47" s="68"/>
-      <c r="C47" s="152" t="s">
+      <c r="C47" s="147" t="s">
         <v>126</v>
       </c>
-      <c r="D47" s="152"/>
-      <c r="E47" s="152"/>
-      <c r="F47" s="152"/>
-      <c r="G47" s="152"/>
-      <c r="H47" s="152"/>
-      <c r="I47" s="152"/>
-      <c r="J47" s="152"/>
-      <c r="K47" s="152"/>
+      <c r="D47" s="147"/>
+      <c r="E47" s="147"/>
+      <c r="F47" s="147"/>
+      <c r="G47" s="147"/>
+      <c r="H47" s="147"/>
+      <c r="I47" s="147"/>
+      <c r="J47" s="147"/>
+      <c r="K47" s="147"/>
     </row>
     <row r="48" spans="1:11" s="71" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="153"/>
-      <c r="B48" s="149" t="s">
+      <c r="A48" s="148"/>
+      <c r="B48" s="144" t="s">
         <v>127</v>
       </c>
-      <c r="C48" s="149" t="s">
+      <c r="C48" s="144" t="s">
         <v>128</v>
       </c>
-      <c r="D48" s="149" t="s">
+      <c r="D48" s="144" t="s">
         <v>129</v>
       </c>
-      <c r="E48" s="149" t="s">
+      <c r="E48" s="144" t="s">
         <v>98</v>
       </c>
-      <c r="F48" s="149" t="s">
+      <c r="F48" s="144" t="s">
         <v>130</v>
       </c>
-      <c r="G48" s="149" t="s">
+      <c r="G48" s="144" t="s">
         <v>102</v>
       </c>
-      <c r="H48" s="154" t="s">
+      <c r="H48" s="149" t="s">
         <v>131</v>
       </c>
-      <c r="I48" s="154"/>
-      <c r="J48" s="154"/>
-      <c r="K48" s="154"/>
+      <c r="I48" s="149"/>
+      <c r="J48" s="149"/>
+      <c r="K48" s="149"/>
     </row>
     <row r="49" spans="1:11" s="71" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="153"/>
-      <c r="B49" s="149"/>
-      <c r="C49" s="149"/>
-      <c r="D49" s="149"/>
-      <c r="E49" s="149"/>
-      <c r="F49" s="149"/>
-      <c r="G49" s="149"/>
-      <c r="H49" s="149" t="s">
+      <c r="A49" s="148"/>
+      <c r="B49" s="144"/>
+      <c r="C49" s="144"/>
+      <c r="D49" s="144"/>
+      <c r="E49" s="144"/>
+      <c r="F49" s="144"/>
+      <c r="G49" s="144"/>
+      <c r="H49" s="144" t="s">
         <v>132</v>
       </c>
-      <c r="I49" s="149"/>
+      <c r="I49" s="144"/>
       <c r="J49" s="70" t="s">
         <v>133</v>
       </c>
@@ -10826,8 +10826,8 @@
       <c r="G50" s="75" t="s">
         <v>103</v>
       </c>
-      <c r="H50" s="150"/>
-      <c r="I50" s="150"/>
+      <c r="H50" s="145"/>
+      <c r="I50" s="145"/>
       <c r="J50" s="77" t="s">
         <v>227</v>
       </c>
@@ -10990,8 +10990,8 @@
         <v>#VALUE!</v>
       </c>
       <c r="G59" s="75"/>
-      <c r="H59" s="150"/>
-      <c r="I59" s="150"/>
+      <c r="H59" s="145"/>
+      <c r="I59" s="145"/>
       <c r="J59" s="77"/>
       <c r="K59" s="77"/>
     </row>
@@ -11006,13 +11006,19 @@
         <v>#VALUE!</v>
       </c>
       <c r="G60" s="75"/>
-      <c r="H60" s="150"/>
-      <c r="I60" s="150"/>
+      <c r="H60" s="145"/>
+      <c r="I60" s="145"/>
       <c r="J60" s="77"/>
       <c r="K60" s="77"/>
     </row>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="A44:K44"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="D33:E33"/>
+    <mergeCell ref="A41:K41"/>
+    <mergeCell ref="A42:K42"/>
+    <mergeCell ref="A43:K43"/>
     <mergeCell ref="H49:I49"/>
     <mergeCell ref="H50:I50"/>
     <mergeCell ref="H59:I59"/>
@@ -11027,12 +11033,6 @@
     <mergeCell ref="F48:F49"/>
     <mergeCell ref="G48:G49"/>
     <mergeCell ref="H48:K48"/>
-    <mergeCell ref="A44:K44"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="D33:E33"/>
-    <mergeCell ref="A41:K41"/>
-    <mergeCell ref="A42:K42"/>
-    <mergeCell ref="A43:K43"/>
   </mergeCells>
   <conditionalFormatting sqref="F50:F60">
     <cfRule type="cellIs" dxfId="2" priority="8" stopIfTrue="1" operator="equal">

</xml_diff>

<commit_message>
Correção no nome dos casos de uso dentro de Product Backlog
</commit_message>
<xml_diff>
--- a/6.Gerenciamento de Projeto/BRA - Planejamento e Controle do Projeto.xlsx
+++ b/6.Gerenciamento de Projeto/BRA - Planejamento e Controle do Projeto.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\fabioas\Development\bra-brasileirao_analyst\6.Gerenciamento de Projeto\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{901D9FD3-C3D1-423C-9CDD-B31180BC1C80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBDB9E48-34D9-4AE1-A170-D0BEA21990C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-19310" yWindow="-110" windowWidth="19420" windowHeight="11020" activeTab="3" xr2:uid="{31237A52-FFD1-4E1D-B5BB-391D11929C61}"/>
+    <workbookView xWindow="-19310" yWindow="-110" windowWidth="19420" windowHeight="11020" activeTab="1" xr2:uid="{31237A52-FFD1-4E1D-B5BB-391D11929C61}"/>
   </bookViews>
   <sheets>
     <sheet name="Equipe" sheetId="1" r:id="rId1"/>
@@ -5464,9 +5464,6 @@
     <t>Fazer login</t>
   </si>
   <si>
-    <t>Ver estatísticas do atleta</t>
-  </si>
-  <si>
     <t>Favoritar atleta</t>
   </si>
   <si>
@@ -5598,21 +5595,6 @@
   </si>
   <si>
     <r>
-      <t xml:space="preserve">Projetar testes para </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>UC 04 - Ver estatísticas do atleta</t>
-    </r>
-  </si>
-  <si>
-    <r>
       <t xml:space="preserve">Modelar, Implementar e Testar o </t>
     </r>
     <r>
@@ -5772,6 +5754,24 @@
   </si>
   <si>
     <t>Entregue</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Projetar testes para </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>UC 04 - Ver estatísticas dos atletas</t>
+    </r>
+  </si>
+  <si>
+    <t>Ver estatísticas dos atletas</t>
   </si>
 </sst>
 </file>
@@ -6749,6 +6749,21 @@
     <xf numFmtId="164" fontId="20" fillId="5" borderId="7" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="28" fillId="12" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="29" fillId="13" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="29" fillId="10" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="28" fillId="3" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="28" fillId="14" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="164" fontId="29" fillId="15" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -6762,21 +6777,6 @@
     <xf numFmtId="0" fontId="0" fillId="15" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="29" fillId="15" borderId="4" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="28" fillId="12" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="29" fillId="13" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="29" fillId="10" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="28" fillId="3" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="28" fillId="14" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="16" fillId="13" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -8713,7 +8713,7 @@
     </row>
     <row r="2" spans="1:3" ht="24.6" x14ac:dyDescent="0.3">
       <c r="A2" s="135" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B2" s="135"/>
       <c r="C2" s="135"/>
@@ -8734,10 +8734,10 @@
         <v>4</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C4" s="115" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
@@ -8745,10 +8745,10 @@
         <v>5</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C5" s="115" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
@@ -8756,10 +8756,10 @@
         <v>6</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C6" s="115" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
@@ -9034,7 +9034,7 @@
         <v>3</v>
       </c>
       <c r="G7" s="12" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="H7" s="15">
         <v>8</v>
@@ -9070,7 +9070,7 @@
         <v>4</v>
       </c>
       <c r="G8" s="12" t="s">
-        <v>212</v>
+        <v>252</v>
       </c>
       <c r="H8" s="15">
         <v>10</v>
@@ -9106,7 +9106,7 @@
         <v>5</v>
       </c>
       <c r="G9" s="12" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="H9" s="15">
         <v>7</v>
@@ -9142,7 +9142,7 @@
         <v>6</v>
       </c>
       <c r="G10" s="12" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="H10" s="15">
         <v>9</v>
@@ -9208,7 +9208,7 @@
         <v>30</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D13" s="13">
         <v>5</v>
@@ -9229,7 +9229,7 @@
         <v>30</v>
       </c>
       <c r="C14" s="12" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D14" s="13">
         <v>2</v>
@@ -9250,7 +9250,7 @@
         <v>30</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="D15" s="13">
         <v>8</v>
@@ -9271,7 +9271,7 @@
         <v>30</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="D16" s="13">
         <v>0.5</v>
@@ -9292,7 +9292,7 @@
         <v>30</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="D17" s="13">
         <v>1</v>
@@ -9334,7 +9334,7 @@
         <v>30</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="D19" s="13">
         <v>8</v>
@@ -9353,7 +9353,7 @@
         <v>30</v>
       </c>
       <c r="C20" s="12" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="D20" s="13">
         <v>2</v>
@@ -9372,7 +9372,7 @@
         <v>30</v>
       </c>
       <c r="C21" s="18" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="D21" s="13">
         <v>1</v>
@@ -9449,7 +9449,7 @@
         <v>35</v>
       </c>
       <c r="C26" s="12" t="s">
-        <v>237</v>
+        <v>251</v>
       </c>
       <c r="D26" s="13">
         <v>1</v>
@@ -9463,7 +9463,7 @@
         <v>35</v>
       </c>
       <c r="C27" s="12" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="D27" s="13">
         <v>20</v>
@@ -9477,7 +9477,7 @@
         <v>35</v>
       </c>
       <c r="C28" s="12" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="D28" s="13">
         <v>1</v>
@@ -9491,7 +9491,7 @@
         <v>35</v>
       </c>
       <c r="C29" s="12" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="D29" s="13">
         <v>20</v>
@@ -9505,7 +9505,7 @@
         <v>35</v>
       </c>
       <c r="C30" s="12" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="D30" s="13">
         <v>1</v>
@@ -9519,7 +9519,7 @@
         <v>35</v>
       </c>
       <c r="C31" s="12" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="D31" s="13">
         <v>8</v>
@@ -9533,7 +9533,7 @@
         <v>35</v>
       </c>
       <c r="C32" s="12" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D32" s="13">
         <v>2</v>
@@ -9547,7 +9547,7 @@
         <v>35</v>
       </c>
       <c r="C33" s="12" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D33" s="13">
         <v>8</v>
@@ -9561,7 +9561,7 @@
         <v>35</v>
       </c>
       <c r="C34" s="12" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="D34" s="13">
         <v>2</v>
@@ -9575,7 +9575,7 @@
         <v>35</v>
       </c>
       <c r="C35" s="12" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="D35" s="13">
         <v>5</v>
@@ -9684,7 +9684,7 @@
         <v>36</v>
       </c>
       <c r="C43" s="12" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="D43" s="13">
         <v>5</v>
@@ -10117,7 +10117,7 @@
         <v>1</v>
       </c>
       <c r="B5" s="116" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="C5" s="117">
         <v>46252</v>
@@ -10129,7 +10129,7 @@
         <v>10.5</v>
       </c>
       <c r="F5" s="119" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="G5" s="117">
         <v>46252</v>
@@ -10144,7 +10144,7 @@
         <v>0</v>
       </c>
       <c r="K5" s="121" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="27.6" x14ac:dyDescent="0.3">
@@ -10152,7 +10152,7 @@
         <v>2</v>
       </c>
       <c r="B6" s="116" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="C6" s="117">
         <v>46273</v>
@@ -10177,7 +10177,7 @@
         <v>3</v>
       </c>
       <c r="B7" s="116" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="C7" s="117">
         <v>46294</v>
@@ -10202,7 +10202,7 @@
         <v>4</v>
       </c>
       <c r="B8" s="124" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="C8" s="125">
         <v>46315</v>
@@ -10610,10 +10610,10 @@
       </c>
     </row>
     <row r="33" spans="1:11" ht="22.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D33" s="151" t="s">
+      <c r="D33" s="145" t="s">
         <v>113</v>
       </c>
-      <c r="E33" s="151"/>
+      <c r="E33" s="145"/>
     </row>
     <row r="34" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="D34" s="63">
@@ -10665,137 +10665,137 @@
     </row>
     <row r="40" spans="1:11" ht="8.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="41" spans="1:11" s="60" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="152" t="s">
+      <c r="A41" s="146" t="s">
         <v>120</v>
       </c>
-      <c r="B41" s="152"/>
-      <c r="C41" s="152"/>
-      <c r="D41" s="152"/>
-      <c r="E41" s="152"/>
-      <c r="F41" s="152"/>
-      <c r="G41" s="152"/>
-      <c r="H41" s="152"/>
-      <c r="I41" s="152"/>
-      <c r="J41" s="152"/>
-      <c r="K41" s="152"/>
+      <c r="B41" s="146"/>
+      <c r="C41" s="146"/>
+      <c r="D41" s="146"/>
+      <c r="E41" s="146"/>
+      <c r="F41" s="146"/>
+      <c r="G41" s="146"/>
+      <c r="H41" s="146"/>
+      <c r="I41" s="146"/>
+      <c r="J41" s="146"/>
+      <c r="K41" s="146"/>
     </row>
     <row r="42" spans="1:11" s="60" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="153" t="s">
+      <c r="A42" s="147" t="s">
         <v>121</v>
       </c>
-      <c r="B42" s="153"/>
-      <c r="C42" s="153"/>
-      <c r="D42" s="153"/>
-      <c r="E42" s="153"/>
-      <c r="F42" s="153"/>
-      <c r="G42" s="153"/>
-      <c r="H42" s="153"/>
-      <c r="I42" s="153"/>
-      <c r="J42" s="153"/>
-      <c r="K42" s="153"/>
+      <c r="B42" s="147"/>
+      <c r="C42" s="147"/>
+      <c r="D42" s="147"/>
+      <c r="E42" s="147"/>
+      <c r="F42" s="147"/>
+      <c r="G42" s="147"/>
+      <c r="H42" s="147"/>
+      <c r="I42" s="147"/>
+      <c r="J42" s="147"/>
+      <c r="K42" s="147"/>
     </row>
     <row r="43" spans="1:11" s="60" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="154" t="s">
+      <c r="A43" s="148" t="s">
         <v>122</v>
       </c>
-      <c r="B43" s="154"/>
-      <c r="C43" s="154"/>
-      <c r="D43" s="154"/>
-      <c r="E43" s="154"/>
-      <c r="F43" s="154"/>
-      <c r="G43" s="154"/>
-      <c r="H43" s="154"/>
-      <c r="I43" s="154"/>
-      <c r="J43" s="154"/>
-      <c r="K43" s="154"/>
+      <c r="B43" s="148"/>
+      <c r="C43" s="148"/>
+      <c r="D43" s="148"/>
+      <c r="E43" s="148"/>
+      <c r="F43" s="148"/>
+      <c r="G43" s="148"/>
+      <c r="H43" s="148"/>
+      <c r="I43" s="148"/>
+      <c r="J43" s="148"/>
+      <c r="K43" s="148"/>
     </row>
     <row r="44" spans="1:11" s="60" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="150" t="s">
+      <c r="A44" s="144" t="s">
         <v>123</v>
       </c>
-      <c r="B44" s="150"/>
-      <c r="C44" s="150"/>
-      <c r="D44" s="150"/>
-      <c r="E44" s="150"/>
-      <c r="F44" s="150"/>
-      <c r="G44" s="150"/>
-      <c r="H44" s="150"/>
-      <c r="I44" s="150"/>
-      <c r="J44" s="150"/>
-      <c r="K44" s="150"/>
+      <c r="B44" s="144"/>
+      <c r="C44" s="144"/>
+      <c r="D44" s="144"/>
+      <c r="E44" s="144"/>
+      <c r="F44" s="144"/>
+      <c r="G44" s="144"/>
+      <c r="H44" s="144"/>
+      <c r="I44" s="144"/>
+      <c r="J44" s="144"/>
+      <c r="K44" s="144"/>
     </row>
     <row r="45" spans="1:11" ht="9" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="46" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A46" s="146" t="s">
+      <c r="A46" s="151" t="s">
         <v>124</v>
       </c>
-      <c r="B46" s="146"/>
-      <c r="C46" s="146"/>
-      <c r="D46" s="146"/>
-      <c r="E46" s="146"/>
-      <c r="F46" s="146"/>
-      <c r="G46" s="146"/>
-      <c r="H46" s="146"/>
-      <c r="I46" s="146"/>
-      <c r="J46" s="146"/>
-      <c r="K46" s="146"/>
+      <c r="B46" s="151"/>
+      <c r="C46" s="151"/>
+      <c r="D46" s="151"/>
+      <c r="E46" s="151"/>
+      <c r="F46" s="151"/>
+      <c r="G46" s="151"/>
+      <c r="H46" s="151"/>
+      <c r="I46" s="151"/>
+      <c r="J46" s="151"/>
+      <c r="K46" s="151"/>
     </row>
     <row r="47" spans="1:11" s="69" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="67" t="s">
         <v>125</v>
       </c>
       <c r="B47" s="68"/>
-      <c r="C47" s="147" t="s">
+      <c r="C47" s="152" t="s">
         <v>126</v>
       </c>
-      <c r="D47" s="147"/>
-      <c r="E47" s="147"/>
-      <c r="F47" s="147"/>
-      <c r="G47" s="147"/>
-      <c r="H47" s="147"/>
-      <c r="I47" s="147"/>
-      <c r="J47" s="147"/>
-      <c r="K47" s="147"/>
+      <c r="D47" s="152"/>
+      <c r="E47" s="152"/>
+      <c r="F47" s="152"/>
+      <c r="G47" s="152"/>
+      <c r="H47" s="152"/>
+      <c r="I47" s="152"/>
+      <c r="J47" s="152"/>
+      <c r="K47" s="152"/>
     </row>
     <row r="48" spans="1:11" s="71" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="148"/>
-      <c r="B48" s="144" t="s">
+      <c r="A48" s="153"/>
+      <c r="B48" s="149" t="s">
         <v>127</v>
       </c>
-      <c r="C48" s="144" t="s">
+      <c r="C48" s="149" t="s">
         <v>128</v>
       </c>
-      <c r="D48" s="144" t="s">
+      <c r="D48" s="149" t="s">
         <v>129</v>
       </c>
-      <c r="E48" s="144" t="s">
+      <c r="E48" s="149" t="s">
         <v>98</v>
       </c>
-      <c r="F48" s="144" t="s">
+      <c r="F48" s="149" t="s">
         <v>130</v>
       </c>
-      <c r="G48" s="144" t="s">
+      <c r="G48" s="149" t="s">
         <v>102</v>
       </c>
-      <c r="H48" s="149" t="s">
+      <c r="H48" s="154" t="s">
         <v>131</v>
       </c>
-      <c r="I48" s="149"/>
-      <c r="J48" s="149"/>
-      <c r="K48" s="149"/>
+      <c r="I48" s="154"/>
+      <c r="J48" s="154"/>
+      <c r="K48" s="154"/>
     </row>
     <row r="49" spans="1:11" s="71" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="148"/>
-      <c r="B49" s="144"/>
-      <c r="C49" s="144"/>
-      <c r="D49" s="144"/>
-      <c r="E49" s="144"/>
-      <c r="F49" s="144"/>
-      <c r="G49" s="144"/>
-      <c r="H49" s="144" t="s">
+      <c r="A49" s="153"/>
+      <c r="B49" s="149"/>
+      <c r="C49" s="149"/>
+      <c r="D49" s="149"/>
+      <c r="E49" s="149"/>
+      <c r="F49" s="149"/>
+      <c r="G49" s="149"/>
+      <c r="H49" s="149" t="s">
         <v>132</v>
       </c>
-      <c r="I49" s="144"/>
+      <c r="I49" s="149"/>
       <c r="J49" s="70" t="s">
         <v>133</v>
       </c>
@@ -10826,13 +10826,13 @@
       <c r="G50" s="75" t="s">
         <v>103</v>
       </c>
-      <c r="H50" s="145"/>
-      <c r="I50" s="145"/>
+      <c r="H50" s="150"/>
+      <c r="I50" s="150"/>
       <c r="J50" s="77" t="s">
+        <v>226</v>
+      </c>
+      <c r="K50" s="77" t="s">
         <v>227</v>
-      </c>
-      <c r="K50" s="77" t="s">
-        <v>228</v>
       </c>
     </row>
     <row r="51" spans="1:11" s="71" customFormat="1" ht="51" x14ac:dyDescent="0.25">
@@ -10840,7 +10840,7 @@
         <v>2</v>
       </c>
       <c r="B51" s="73" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="C51" s="74">
         <v>46252</v>
@@ -10861,10 +10861,10 @@
       <c r="H51" s="78"/>
       <c r="I51" s="79"/>
       <c r="J51" s="77" t="s">
+        <v>229</v>
+      </c>
+      <c r="K51" s="77" t="s">
         <v>230</v>
-      </c>
-      <c r="K51" s="77" t="s">
-        <v>231</v>
       </c>
     </row>
     <row r="52" spans="1:11" s="71" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -10990,8 +10990,8 @@
         <v>#VALUE!</v>
       </c>
       <c r="G59" s="75"/>
-      <c r="H59" s="145"/>
-      <c r="I59" s="145"/>
+      <c r="H59" s="150"/>
+      <c r="I59" s="150"/>
       <c r="J59" s="77"/>
       <c r="K59" s="77"/>
     </row>
@@ -11006,19 +11006,13 @@
         <v>#VALUE!</v>
       </c>
       <c r="G60" s="75"/>
-      <c r="H60" s="145"/>
-      <c r="I60" s="145"/>
+      <c r="H60" s="150"/>
+      <c r="I60" s="150"/>
       <c r="J60" s="77"/>
       <c r="K60" s="77"/>
     </row>
   </sheetData>
   <mergeCells count="20">
-    <mergeCell ref="A44:K44"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="D33:E33"/>
-    <mergeCell ref="A41:K41"/>
-    <mergeCell ref="A42:K42"/>
-    <mergeCell ref="A43:K43"/>
     <mergeCell ref="H49:I49"/>
     <mergeCell ref="H50:I50"/>
     <mergeCell ref="H59:I59"/>
@@ -11033,6 +11027,12 @@
     <mergeCell ref="F48:F49"/>
     <mergeCell ref="G48:G49"/>
     <mergeCell ref="H48:K48"/>
+    <mergeCell ref="A44:K44"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="D33:E33"/>
+    <mergeCell ref="A41:K41"/>
+    <mergeCell ref="A42:K42"/>
+    <mergeCell ref="A43:K43"/>
   </mergeCells>
   <conditionalFormatting sqref="F50:F60">
     <cfRule type="cellIs" dxfId="2" priority="8" stopIfTrue="1" operator="equal">

</xml_diff>